<commit_message>
Ajoute l'onglet Modèles à la flotte et génère la page du site à partir de ces fiches
Flotte > Modèles : marque, modèle, type (filtre du site), gamme, boîte,
carburant, places, portes, valises, prix, km supplémentaire, caution,
description et photo (recadrée en 1200 × 750). Reprise en un clic des 8
modèles déjà présents sur le site. Les véhicules, contrats et factures
utilisent désormais ces fiches.

outils/catalogue.mjs régénère la section « Notre flotte », le JSON-LD et
llms.txt depuis Firestore ; un workflow GitHub le lance toutes les 15
minutes et ne commite que s'il y a un changement. Le site reste statique.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PgtSFbTj6XziR1xBRYkS6p
</commit_message>
<xml_diff>
--- a/backoffice/modele-import-flotte.xlsx
+++ b/backoffice/modele-import-flotte.xlsx
@@ -4442,13 +4442,13 @@
     </row>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez un modèle de la liste (onglet Listes)." type="list">
+    <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Modèle absent de la liste : vérifiez qu'il existe dans le back-office (Flotte &gt; Modèles)." type="list" errorStyle="warning">
       <formula1>=Listes!$A$2:$A$9</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez un statut de la liste." type="list">
+    <dataValidation sqref="H2:H501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez un statut de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$B$2:$B$5</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez un carburant de la liste." type="list">
+    <dataValidation sqref="E2:E501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez un carburant de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$C$2:$C$5</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F501 M2:N501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Nombre entier de kilomètres." type="whole" operator="between">

</xml_diff>

<commit_message>
Back-office : tableau de bord en page d'accueil
Départs et retours du jour, réservations à confirmer, confirmées à livrer
(avec blocage de paiement), contrats en cours et retards, contrats non
réglés, répartition de la flotte, véhicules indisponibles, documents
administratifs à renouveler sous 30 jours et entretiens à prévoir. Chaque
indicateur ouvre la liste filtrée correspondante.

Ajoute la date d'autorisation de circulation aux véhicules (fiche, import
Excel, démonstration) et un filtre « À livrer » dans les réservations.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PgtSFbTj6XziR1xBRYkS6p
</commit_message>
<xml_diff>
--- a/backoffice/modele-import-flotte.xlsx
+++ b/backoffice/modele-import-flotte.xlsx
@@ -231,10 +231,15 @@
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
+        <t>Date au format jj/mm/aaaa.</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
         <t>Vide = 10 000 km.</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>Vide = 40 000 km.</t>
       </text>
@@ -532,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -550,6 +555,7 @@
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -708,15 +714,20 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
+          <t>Autorisation de circulation jusqu'au</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
           <t>Vidange tous les (km)</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>Pneus tous les (km)</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr">
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -771,13 +782,18 @@
           <t>31/01/2027</t>
         </is>
       </c>
-      <c r="M17" s="5" t="n">
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>30/09/2027</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="n">
         <v>10000</v>
       </c>
-      <c r="N17" s="5" t="n">
+      <c r="O17" s="5" t="n">
         <v>40000</v>
       </c>
-      <c r="O17" s="5" t="inlineStr"/>
+      <c r="P17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -823,7 +839,11 @@
           <t>01/02/2027</t>
         </is>
       </c>
-      <c r="L18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>31/05/2027</t>
+        </is>
+      </c>
       <c r="M18" s="5" t="inlineStr"/>
       <c r="N18" s="5" t="inlineStr"/>
       <c r="O18" s="5" t="inlineStr">
@@ -843,7 +863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O501"/>
+  <dimension ref="A1:P501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -858,9 +878,10 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -926,15 +947,20 @@
       </c>
       <c r="M1" s="6" t="inlineStr">
         <is>
+          <t>Autorisation de circulation jusqu'au</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
           <t>Vidange tous les (km)</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Pneus tous les (km)</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -946,6 +972,7 @@
       <c r="J2" s="8" t="n"/>
       <c r="K2" s="8" t="n"/>
       <c r="L2" s="8" t="n"/>
+      <c r="M2" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="F3" s="7" t="n"/>
@@ -953,6 +980,7 @@
       <c r="J3" s="8" t="n"/>
       <c r="K3" s="8" t="n"/>
       <c r="L3" s="8" t="n"/>
+      <c r="M3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="F4" s="7" t="n"/>
@@ -960,6 +988,7 @@
       <c r="J4" s="8" t="n"/>
       <c r="K4" s="8" t="n"/>
       <c r="L4" s="8" t="n"/>
+      <c r="M4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="F5" s="7" t="n"/>
@@ -967,6 +996,7 @@
       <c r="J5" s="8" t="n"/>
       <c r="K5" s="8" t="n"/>
       <c r="L5" s="8" t="n"/>
+      <c r="M5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="F6" s="7" t="n"/>
@@ -974,6 +1004,7 @@
       <c r="J6" s="8" t="n"/>
       <c r="K6" s="8" t="n"/>
       <c r="L6" s="8" t="n"/>
+      <c r="M6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="F7" s="7" t="n"/>
@@ -981,6 +1012,7 @@
       <c r="J7" s="8" t="n"/>
       <c r="K7" s="8" t="n"/>
       <c r="L7" s="8" t="n"/>
+      <c r="M7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="F8" s="7" t="n"/>
@@ -988,6 +1020,7 @@
       <c r="J8" s="8" t="n"/>
       <c r="K8" s="8" t="n"/>
       <c r="L8" s="8" t="n"/>
+      <c r="M8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="F9" s="7" t="n"/>
@@ -995,6 +1028,7 @@
       <c r="J9" s="8" t="n"/>
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="n"/>
+      <c r="M9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="F10" s="7" t="n"/>
@@ -1002,6 +1036,7 @@
       <c r="J10" s="8" t="n"/>
       <c r="K10" s="8" t="n"/>
       <c r="L10" s="8" t="n"/>
+      <c r="M10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="F11" s="7" t="n"/>
@@ -1009,6 +1044,7 @@
       <c r="J11" s="8" t="n"/>
       <c r="K11" s="8" t="n"/>
       <c r="L11" s="8" t="n"/>
+      <c r="M11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="F12" s="7" t="n"/>
@@ -1016,6 +1052,7 @@
       <c r="J12" s="8" t="n"/>
       <c r="K12" s="8" t="n"/>
       <c r="L12" s="8" t="n"/>
+      <c r="M12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="F13" s="7" t="n"/>
@@ -1023,6 +1060,7 @@
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>
       <c r="L13" s="8" t="n"/>
+      <c r="M13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="F14" s="7" t="n"/>
@@ -1030,6 +1068,7 @@
       <c r="J14" s="8" t="n"/>
       <c r="K14" s="8" t="n"/>
       <c r="L14" s="8" t="n"/>
+      <c r="M14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="F15" s="7" t="n"/>
@@ -1037,6 +1076,7 @@
       <c r="J15" s="8" t="n"/>
       <c r="K15" s="8" t="n"/>
       <c r="L15" s="8" t="n"/>
+      <c r="M15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="F16" s="7" t="n"/>
@@ -1044,6 +1084,7 @@
       <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="n"/>
+      <c r="M16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="F17" s="7" t="n"/>
@@ -1051,6 +1092,7 @@
       <c r="J17" s="8" t="n"/>
       <c r="K17" s="8" t="n"/>
       <c r="L17" s="8" t="n"/>
+      <c r="M17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="F18" s="7" t="n"/>
@@ -1058,6 +1100,7 @@
       <c r="J18" s="8" t="n"/>
       <c r="K18" s="8" t="n"/>
       <c r="L18" s="8" t="n"/>
+      <c r="M18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="F19" s="7" t="n"/>
@@ -1065,6 +1108,7 @@
       <c r="J19" s="8" t="n"/>
       <c r="K19" s="8" t="n"/>
       <c r="L19" s="8" t="n"/>
+      <c r="M19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="F20" s="7" t="n"/>
@@ -1072,6 +1116,7 @@
       <c r="J20" s="8" t="n"/>
       <c r="K20" s="8" t="n"/>
       <c r="L20" s="8" t="n"/>
+      <c r="M20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="F21" s="7" t="n"/>
@@ -1079,6 +1124,7 @@
       <c r="J21" s="8" t="n"/>
       <c r="K21" s="8" t="n"/>
       <c r="L21" s="8" t="n"/>
+      <c r="M21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="F22" s="7" t="n"/>
@@ -1086,6 +1132,7 @@
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
       <c r="L22" s="8" t="n"/>
+      <c r="M22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="F23" s="7" t="n"/>
@@ -1093,6 +1140,7 @@
       <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
       <c r="L23" s="8" t="n"/>
+      <c r="M23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="F24" s="7" t="n"/>
@@ -1100,6 +1148,7 @@
       <c r="J24" s="8" t="n"/>
       <c r="K24" s="8" t="n"/>
       <c r="L24" s="8" t="n"/>
+      <c r="M24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="F25" s="7" t="n"/>
@@ -1107,6 +1156,7 @@
       <c r="J25" s="8" t="n"/>
       <c r="K25" s="8" t="n"/>
       <c r="L25" s="8" t="n"/>
+      <c r="M25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="F26" s="7" t="n"/>
@@ -1114,6 +1164,7 @@
       <c r="J26" s="8" t="n"/>
       <c r="K26" s="8" t="n"/>
       <c r="L26" s="8" t="n"/>
+      <c r="M26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="F27" s="7" t="n"/>
@@ -1121,6 +1172,7 @@
       <c r="J27" s="8" t="n"/>
       <c r="K27" s="8" t="n"/>
       <c r="L27" s="8" t="n"/>
+      <c r="M27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="F28" s="7" t="n"/>
@@ -1128,6 +1180,7 @@
       <c r="J28" s="8" t="n"/>
       <c r="K28" s="8" t="n"/>
       <c r="L28" s="8" t="n"/>
+      <c r="M28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="F29" s="7" t="n"/>
@@ -1135,6 +1188,7 @@
       <c r="J29" s="8" t="n"/>
       <c r="K29" s="8" t="n"/>
       <c r="L29" s="8" t="n"/>
+      <c r="M29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="F30" s="7" t="n"/>
@@ -1142,6 +1196,7 @@
       <c r="J30" s="8" t="n"/>
       <c r="K30" s="8" t="n"/>
       <c r="L30" s="8" t="n"/>
+      <c r="M30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="F31" s="7" t="n"/>
@@ -1149,6 +1204,7 @@
       <c r="J31" s="8" t="n"/>
       <c r="K31" s="8" t="n"/>
       <c r="L31" s="8" t="n"/>
+      <c r="M31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="F32" s="7" t="n"/>
@@ -1156,6 +1212,7 @@
       <c r="J32" s="8" t="n"/>
       <c r="K32" s="8" t="n"/>
       <c r="L32" s="8" t="n"/>
+      <c r="M32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="F33" s="7" t="n"/>
@@ -1163,6 +1220,7 @@
       <c r="J33" s="8" t="n"/>
       <c r="K33" s="8" t="n"/>
       <c r="L33" s="8" t="n"/>
+      <c r="M33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="F34" s="7" t="n"/>
@@ -1170,6 +1228,7 @@
       <c r="J34" s="8" t="n"/>
       <c r="K34" s="8" t="n"/>
       <c r="L34" s="8" t="n"/>
+      <c r="M34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="F35" s="7" t="n"/>
@@ -1177,6 +1236,7 @@
       <c r="J35" s="8" t="n"/>
       <c r="K35" s="8" t="n"/>
       <c r="L35" s="8" t="n"/>
+      <c r="M35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="F36" s="7" t="n"/>
@@ -1184,6 +1244,7 @@
       <c r="J36" s="8" t="n"/>
       <c r="K36" s="8" t="n"/>
       <c r="L36" s="8" t="n"/>
+      <c r="M36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="F37" s="7" t="n"/>
@@ -1191,6 +1252,7 @@
       <c r="J37" s="8" t="n"/>
       <c r="K37" s="8" t="n"/>
       <c r="L37" s="8" t="n"/>
+      <c r="M37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="F38" s="7" t="n"/>
@@ -1198,6 +1260,7 @@
       <c r="J38" s="8" t="n"/>
       <c r="K38" s="8" t="n"/>
       <c r="L38" s="8" t="n"/>
+      <c r="M38" s="8" t="n"/>
     </row>
     <row r="39">
       <c r="F39" s="7" t="n"/>
@@ -1205,6 +1268,7 @@
       <c r="J39" s="8" t="n"/>
       <c r="K39" s="8" t="n"/>
       <c r="L39" s="8" t="n"/>
+      <c r="M39" s="8" t="n"/>
     </row>
     <row r="40">
       <c r="F40" s="7" t="n"/>
@@ -1212,6 +1276,7 @@
       <c r="J40" s="8" t="n"/>
       <c r="K40" s="8" t="n"/>
       <c r="L40" s="8" t="n"/>
+      <c r="M40" s="8" t="n"/>
     </row>
     <row r="41">
       <c r="F41" s="7" t="n"/>
@@ -1219,6 +1284,7 @@
       <c r="J41" s="8" t="n"/>
       <c r="K41" s="8" t="n"/>
       <c r="L41" s="8" t="n"/>
+      <c r="M41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="F42" s="7" t="n"/>
@@ -1226,6 +1292,7 @@
       <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>
       <c r="L42" s="8" t="n"/>
+      <c r="M42" s="8" t="n"/>
     </row>
     <row r="43">
       <c r="F43" s="7" t="n"/>
@@ -1233,6 +1300,7 @@
       <c r="J43" s="8" t="n"/>
       <c r="K43" s="8" t="n"/>
       <c r="L43" s="8" t="n"/>
+      <c r="M43" s="8" t="n"/>
     </row>
     <row r="44">
       <c r="F44" s="7" t="n"/>
@@ -1240,6 +1308,7 @@
       <c r="J44" s="8" t="n"/>
       <c r="K44" s="8" t="n"/>
       <c r="L44" s="8" t="n"/>
+      <c r="M44" s="8" t="n"/>
     </row>
     <row r="45">
       <c r="F45" s="7" t="n"/>
@@ -1247,6 +1316,7 @@
       <c r="J45" s="8" t="n"/>
       <c r="K45" s="8" t="n"/>
       <c r="L45" s="8" t="n"/>
+      <c r="M45" s="8" t="n"/>
     </row>
     <row r="46">
       <c r="F46" s="7" t="n"/>
@@ -1254,6 +1324,7 @@
       <c r="J46" s="8" t="n"/>
       <c r="K46" s="8" t="n"/>
       <c r="L46" s="8" t="n"/>
+      <c r="M46" s="8" t="n"/>
     </row>
     <row r="47">
       <c r="F47" s="7" t="n"/>
@@ -1261,6 +1332,7 @@
       <c r="J47" s="8" t="n"/>
       <c r="K47" s="8" t="n"/>
       <c r="L47" s="8" t="n"/>
+      <c r="M47" s="8" t="n"/>
     </row>
     <row r="48">
       <c r="F48" s="7" t="n"/>
@@ -1268,6 +1340,7 @@
       <c r="J48" s="8" t="n"/>
       <c r="K48" s="8" t="n"/>
       <c r="L48" s="8" t="n"/>
+      <c r="M48" s="8" t="n"/>
     </row>
     <row r="49">
       <c r="F49" s="7" t="n"/>
@@ -1275,6 +1348,7 @@
       <c r="J49" s="8" t="n"/>
       <c r="K49" s="8" t="n"/>
       <c r="L49" s="8" t="n"/>
+      <c r="M49" s="8" t="n"/>
     </row>
     <row r="50">
       <c r="F50" s="7" t="n"/>
@@ -1282,6 +1356,7 @@
       <c r="J50" s="8" t="n"/>
       <c r="K50" s="8" t="n"/>
       <c r="L50" s="8" t="n"/>
+      <c r="M50" s="8" t="n"/>
     </row>
     <row r="51">
       <c r="F51" s="7" t="n"/>
@@ -1289,6 +1364,7 @@
       <c r="J51" s="8" t="n"/>
       <c r="K51" s="8" t="n"/>
       <c r="L51" s="8" t="n"/>
+      <c r="M51" s="8" t="n"/>
     </row>
     <row r="52">
       <c r="F52" s="7" t="n"/>
@@ -1296,6 +1372,7 @@
       <c r="J52" s="8" t="n"/>
       <c r="K52" s="8" t="n"/>
       <c r="L52" s="8" t="n"/>
+      <c r="M52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="F53" s="7" t="n"/>
@@ -1303,6 +1380,7 @@
       <c r="J53" s="8" t="n"/>
       <c r="K53" s="8" t="n"/>
       <c r="L53" s="8" t="n"/>
+      <c r="M53" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="F54" s="7" t="n"/>
@@ -1310,6 +1388,7 @@
       <c r="J54" s="8" t="n"/>
       <c r="K54" s="8" t="n"/>
       <c r="L54" s="8" t="n"/>
+      <c r="M54" s="8" t="n"/>
     </row>
     <row r="55">
       <c r="F55" s="7" t="n"/>
@@ -1317,6 +1396,7 @@
       <c r="J55" s="8" t="n"/>
       <c r="K55" s="8" t="n"/>
       <c r="L55" s="8" t="n"/>
+      <c r="M55" s="8" t="n"/>
     </row>
     <row r="56">
       <c r="F56" s="7" t="n"/>
@@ -1324,6 +1404,7 @@
       <c r="J56" s="8" t="n"/>
       <c r="K56" s="8" t="n"/>
       <c r="L56" s="8" t="n"/>
+      <c r="M56" s="8" t="n"/>
     </row>
     <row r="57">
       <c r="F57" s="7" t="n"/>
@@ -1331,6 +1412,7 @@
       <c r="J57" s="8" t="n"/>
       <c r="K57" s="8" t="n"/>
       <c r="L57" s="8" t="n"/>
+      <c r="M57" s="8" t="n"/>
     </row>
     <row r="58">
       <c r="F58" s="7" t="n"/>
@@ -1338,6 +1420,7 @@
       <c r="J58" s="8" t="n"/>
       <c r="K58" s="8" t="n"/>
       <c r="L58" s="8" t="n"/>
+      <c r="M58" s="8" t="n"/>
     </row>
     <row r="59">
       <c r="F59" s="7" t="n"/>
@@ -1345,6 +1428,7 @@
       <c r="J59" s="8" t="n"/>
       <c r="K59" s="8" t="n"/>
       <c r="L59" s="8" t="n"/>
+      <c r="M59" s="8" t="n"/>
     </row>
     <row r="60">
       <c r="F60" s="7" t="n"/>
@@ -1352,6 +1436,7 @@
       <c r="J60" s="8" t="n"/>
       <c r="K60" s="8" t="n"/>
       <c r="L60" s="8" t="n"/>
+      <c r="M60" s="8" t="n"/>
     </row>
     <row r="61">
       <c r="F61" s="7" t="n"/>
@@ -1359,6 +1444,7 @@
       <c r="J61" s="8" t="n"/>
       <c r="K61" s="8" t="n"/>
       <c r="L61" s="8" t="n"/>
+      <c r="M61" s="8" t="n"/>
     </row>
     <row r="62">
       <c r="F62" s="7" t="n"/>
@@ -1366,6 +1452,7 @@
       <c r="J62" s="8" t="n"/>
       <c r="K62" s="8" t="n"/>
       <c r="L62" s="8" t="n"/>
+      <c r="M62" s="8" t="n"/>
     </row>
     <row r="63">
       <c r="F63" s="7" t="n"/>
@@ -1373,6 +1460,7 @@
       <c r="J63" s="8" t="n"/>
       <c r="K63" s="8" t="n"/>
       <c r="L63" s="8" t="n"/>
+      <c r="M63" s="8" t="n"/>
     </row>
     <row r="64">
       <c r="F64" s="7" t="n"/>
@@ -1380,6 +1468,7 @@
       <c r="J64" s="8" t="n"/>
       <c r="K64" s="8" t="n"/>
       <c r="L64" s="8" t="n"/>
+      <c r="M64" s="8" t="n"/>
     </row>
     <row r="65">
       <c r="F65" s="7" t="n"/>
@@ -1387,6 +1476,7 @@
       <c r="J65" s="8" t="n"/>
       <c r="K65" s="8" t="n"/>
       <c r="L65" s="8" t="n"/>
+      <c r="M65" s="8" t="n"/>
     </row>
     <row r="66">
       <c r="F66" s="7" t="n"/>
@@ -1394,6 +1484,7 @@
       <c r="J66" s="8" t="n"/>
       <c r="K66" s="8" t="n"/>
       <c r="L66" s="8" t="n"/>
+      <c r="M66" s="8" t="n"/>
     </row>
     <row r="67">
       <c r="F67" s="7" t="n"/>
@@ -1401,6 +1492,7 @@
       <c r="J67" s="8" t="n"/>
       <c r="K67" s="8" t="n"/>
       <c r="L67" s="8" t="n"/>
+      <c r="M67" s="8" t="n"/>
     </row>
     <row r="68">
       <c r="F68" s="7" t="n"/>
@@ -1408,6 +1500,7 @@
       <c r="J68" s="8" t="n"/>
       <c r="K68" s="8" t="n"/>
       <c r="L68" s="8" t="n"/>
+      <c r="M68" s="8" t="n"/>
     </row>
     <row r="69">
       <c r="F69" s="7" t="n"/>
@@ -1415,6 +1508,7 @@
       <c r="J69" s="8" t="n"/>
       <c r="K69" s="8" t="n"/>
       <c r="L69" s="8" t="n"/>
+      <c r="M69" s="8" t="n"/>
     </row>
     <row r="70">
       <c r="F70" s="7" t="n"/>
@@ -1422,6 +1516,7 @@
       <c r="J70" s="8" t="n"/>
       <c r="K70" s="8" t="n"/>
       <c r="L70" s="8" t="n"/>
+      <c r="M70" s="8" t="n"/>
     </row>
     <row r="71">
       <c r="F71" s="7" t="n"/>
@@ -1429,6 +1524,7 @@
       <c r="J71" s="8" t="n"/>
       <c r="K71" s="8" t="n"/>
       <c r="L71" s="8" t="n"/>
+      <c r="M71" s="8" t="n"/>
     </row>
     <row r="72">
       <c r="F72" s="7" t="n"/>
@@ -1436,6 +1532,7 @@
       <c r="J72" s="8" t="n"/>
       <c r="K72" s="8" t="n"/>
       <c r="L72" s="8" t="n"/>
+      <c r="M72" s="8" t="n"/>
     </row>
     <row r="73">
       <c r="F73" s="7" t="n"/>
@@ -1443,6 +1540,7 @@
       <c r="J73" s="8" t="n"/>
       <c r="K73" s="8" t="n"/>
       <c r="L73" s="8" t="n"/>
+      <c r="M73" s="8" t="n"/>
     </row>
     <row r="74">
       <c r="F74" s="7" t="n"/>
@@ -1450,6 +1548,7 @@
       <c r="J74" s="8" t="n"/>
       <c r="K74" s="8" t="n"/>
       <c r="L74" s="8" t="n"/>
+      <c r="M74" s="8" t="n"/>
     </row>
     <row r="75">
       <c r="F75" s="7" t="n"/>
@@ -1457,6 +1556,7 @@
       <c r="J75" s="8" t="n"/>
       <c r="K75" s="8" t="n"/>
       <c r="L75" s="8" t="n"/>
+      <c r="M75" s="8" t="n"/>
     </row>
     <row r="76">
       <c r="F76" s="7" t="n"/>
@@ -1464,6 +1564,7 @@
       <c r="J76" s="8" t="n"/>
       <c r="K76" s="8" t="n"/>
       <c r="L76" s="8" t="n"/>
+      <c r="M76" s="8" t="n"/>
     </row>
     <row r="77">
       <c r="F77" s="7" t="n"/>
@@ -1471,6 +1572,7 @@
       <c r="J77" s="8" t="n"/>
       <c r="K77" s="8" t="n"/>
       <c r="L77" s="8" t="n"/>
+      <c r="M77" s="8" t="n"/>
     </row>
     <row r="78">
       <c r="F78" s="7" t="n"/>
@@ -1478,6 +1580,7 @@
       <c r="J78" s="8" t="n"/>
       <c r="K78" s="8" t="n"/>
       <c r="L78" s="8" t="n"/>
+      <c r="M78" s="8" t="n"/>
     </row>
     <row r="79">
       <c r="F79" s="7" t="n"/>
@@ -1485,6 +1588,7 @@
       <c r="J79" s="8" t="n"/>
       <c r="K79" s="8" t="n"/>
       <c r="L79" s="8" t="n"/>
+      <c r="M79" s="8" t="n"/>
     </row>
     <row r="80">
       <c r="F80" s="7" t="n"/>
@@ -1492,6 +1596,7 @@
       <c r="J80" s="8" t="n"/>
       <c r="K80" s="8" t="n"/>
       <c r="L80" s="8" t="n"/>
+      <c r="M80" s="8" t="n"/>
     </row>
     <row r="81">
       <c r="F81" s="7" t="n"/>
@@ -1499,6 +1604,7 @@
       <c r="J81" s="8" t="n"/>
       <c r="K81" s="8" t="n"/>
       <c r="L81" s="8" t="n"/>
+      <c r="M81" s="8" t="n"/>
     </row>
     <row r="82">
       <c r="F82" s="7" t="n"/>
@@ -1506,6 +1612,7 @@
       <c r="J82" s="8" t="n"/>
       <c r="K82" s="8" t="n"/>
       <c r="L82" s="8" t="n"/>
+      <c r="M82" s="8" t="n"/>
     </row>
     <row r="83">
       <c r="F83" s="7" t="n"/>
@@ -1513,6 +1620,7 @@
       <c r="J83" s="8" t="n"/>
       <c r="K83" s="8" t="n"/>
       <c r="L83" s="8" t="n"/>
+      <c r="M83" s="8" t="n"/>
     </row>
     <row r="84">
       <c r="F84" s="7" t="n"/>
@@ -1520,6 +1628,7 @@
       <c r="J84" s="8" t="n"/>
       <c r="K84" s="8" t="n"/>
       <c r="L84" s="8" t="n"/>
+      <c r="M84" s="8" t="n"/>
     </row>
     <row r="85">
       <c r="F85" s="7" t="n"/>
@@ -1527,6 +1636,7 @@
       <c r="J85" s="8" t="n"/>
       <c r="K85" s="8" t="n"/>
       <c r="L85" s="8" t="n"/>
+      <c r="M85" s="8" t="n"/>
     </row>
     <row r="86">
       <c r="F86" s="7" t="n"/>
@@ -1534,6 +1644,7 @@
       <c r="J86" s="8" t="n"/>
       <c r="K86" s="8" t="n"/>
       <c r="L86" s="8" t="n"/>
+      <c r="M86" s="8" t="n"/>
     </row>
     <row r="87">
       <c r="F87" s="7" t="n"/>
@@ -1541,6 +1652,7 @@
       <c r="J87" s="8" t="n"/>
       <c r="K87" s="8" t="n"/>
       <c r="L87" s="8" t="n"/>
+      <c r="M87" s="8" t="n"/>
     </row>
     <row r="88">
       <c r="F88" s="7" t="n"/>
@@ -1548,6 +1660,7 @@
       <c r="J88" s="8" t="n"/>
       <c r="K88" s="8" t="n"/>
       <c r="L88" s="8" t="n"/>
+      <c r="M88" s="8" t="n"/>
     </row>
     <row r="89">
       <c r="F89" s="7" t="n"/>
@@ -1555,6 +1668,7 @@
       <c r="J89" s="8" t="n"/>
       <c r="K89" s="8" t="n"/>
       <c r="L89" s="8" t="n"/>
+      <c r="M89" s="8" t="n"/>
     </row>
     <row r="90">
       <c r="F90" s="7" t="n"/>
@@ -1562,6 +1676,7 @@
       <c r="J90" s="8" t="n"/>
       <c r="K90" s="8" t="n"/>
       <c r="L90" s="8" t="n"/>
+      <c r="M90" s="8" t="n"/>
     </row>
     <row r="91">
       <c r="F91" s="7" t="n"/>
@@ -1569,6 +1684,7 @@
       <c r="J91" s="8" t="n"/>
       <c r="K91" s="8" t="n"/>
       <c r="L91" s="8" t="n"/>
+      <c r="M91" s="8" t="n"/>
     </row>
     <row r="92">
       <c r="F92" s="7" t="n"/>
@@ -1576,6 +1692,7 @@
       <c r="J92" s="8" t="n"/>
       <c r="K92" s="8" t="n"/>
       <c r="L92" s="8" t="n"/>
+      <c r="M92" s="8" t="n"/>
     </row>
     <row r="93">
       <c r="F93" s="7" t="n"/>
@@ -1583,6 +1700,7 @@
       <c r="J93" s="8" t="n"/>
       <c r="K93" s="8" t="n"/>
       <c r="L93" s="8" t="n"/>
+      <c r="M93" s="8" t="n"/>
     </row>
     <row r="94">
       <c r="F94" s="7" t="n"/>
@@ -1590,6 +1708,7 @@
       <c r="J94" s="8" t="n"/>
       <c r="K94" s="8" t="n"/>
       <c r="L94" s="8" t="n"/>
+      <c r="M94" s="8" t="n"/>
     </row>
     <row r="95">
       <c r="F95" s="7" t="n"/>
@@ -1597,6 +1716,7 @@
       <c r="J95" s="8" t="n"/>
       <c r="K95" s="8" t="n"/>
       <c r="L95" s="8" t="n"/>
+      <c r="M95" s="8" t="n"/>
     </row>
     <row r="96">
       <c r="F96" s="7" t="n"/>
@@ -1604,6 +1724,7 @@
       <c r="J96" s="8" t="n"/>
       <c r="K96" s="8" t="n"/>
       <c r="L96" s="8" t="n"/>
+      <c r="M96" s="8" t="n"/>
     </row>
     <row r="97">
       <c r="F97" s="7" t="n"/>
@@ -1611,6 +1732,7 @@
       <c r="J97" s="8" t="n"/>
       <c r="K97" s="8" t="n"/>
       <c r="L97" s="8" t="n"/>
+      <c r="M97" s="8" t="n"/>
     </row>
     <row r="98">
       <c r="F98" s="7" t="n"/>
@@ -1618,6 +1740,7 @@
       <c r="J98" s="8" t="n"/>
       <c r="K98" s="8" t="n"/>
       <c r="L98" s="8" t="n"/>
+      <c r="M98" s="8" t="n"/>
     </row>
     <row r="99">
       <c r="F99" s="7" t="n"/>
@@ -1625,6 +1748,7 @@
       <c r="J99" s="8" t="n"/>
       <c r="K99" s="8" t="n"/>
       <c r="L99" s="8" t="n"/>
+      <c r="M99" s="8" t="n"/>
     </row>
     <row r="100">
       <c r="F100" s="7" t="n"/>
@@ -1632,6 +1756,7 @@
       <c r="J100" s="8" t="n"/>
       <c r="K100" s="8" t="n"/>
       <c r="L100" s="8" t="n"/>
+      <c r="M100" s="8" t="n"/>
     </row>
     <row r="101">
       <c r="F101" s="7" t="n"/>
@@ -1639,6 +1764,7 @@
       <c r="J101" s="8" t="n"/>
       <c r="K101" s="8" t="n"/>
       <c r="L101" s="8" t="n"/>
+      <c r="M101" s="8" t="n"/>
     </row>
     <row r="102">
       <c r="F102" s="7" t="n"/>
@@ -1646,6 +1772,7 @@
       <c r="J102" s="8" t="n"/>
       <c r="K102" s="8" t="n"/>
       <c r="L102" s="8" t="n"/>
+      <c r="M102" s="8" t="n"/>
     </row>
     <row r="103">
       <c r="F103" s="7" t="n"/>
@@ -1653,6 +1780,7 @@
       <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="n"/>
       <c r="L103" s="8" t="n"/>
+      <c r="M103" s="8" t="n"/>
     </row>
     <row r="104">
       <c r="F104" s="7" t="n"/>
@@ -1660,6 +1788,7 @@
       <c r="J104" s="8" t="n"/>
       <c r="K104" s="8" t="n"/>
       <c r="L104" s="8" t="n"/>
+      <c r="M104" s="8" t="n"/>
     </row>
     <row r="105">
       <c r="F105" s="7" t="n"/>
@@ -1667,6 +1796,7 @@
       <c r="J105" s="8" t="n"/>
       <c r="K105" s="8" t="n"/>
       <c r="L105" s="8" t="n"/>
+      <c r="M105" s="8" t="n"/>
     </row>
     <row r="106">
       <c r="F106" s="7" t="n"/>
@@ -1674,6 +1804,7 @@
       <c r="J106" s="8" t="n"/>
       <c r="K106" s="8" t="n"/>
       <c r="L106" s="8" t="n"/>
+      <c r="M106" s="8" t="n"/>
     </row>
     <row r="107">
       <c r="F107" s="7" t="n"/>
@@ -1681,6 +1812,7 @@
       <c r="J107" s="8" t="n"/>
       <c r="K107" s="8" t="n"/>
       <c r="L107" s="8" t="n"/>
+      <c r="M107" s="8" t="n"/>
     </row>
     <row r="108">
       <c r="F108" s="7" t="n"/>
@@ -1688,6 +1820,7 @@
       <c r="J108" s="8" t="n"/>
       <c r="K108" s="8" t="n"/>
       <c r="L108" s="8" t="n"/>
+      <c r="M108" s="8" t="n"/>
     </row>
     <row r="109">
       <c r="F109" s="7" t="n"/>
@@ -1695,6 +1828,7 @@
       <c r="J109" s="8" t="n"/>
       <c r="K109" s="8" t="n"/>
       <c r="L109" s="8" t="n"/>
+      <c r="M109" s="8" t="n"/>
     </row>
     <row r="110">
       <c r="F110" s="7" t="n"/>
@@ -1702,6 +1836,7 @@
       <c r="J110" s="8" t="n"/>
       <c r="K110" s="8" t="n"/>
       <c r="L110" s="8" t="n"/>
+      <c r="M110" s="8" t="n"/>
     </row>
     <row r="111">
       <c r="F111" s="7" t="n"/>
@@ -1709,6 +1844,7 @@
       <c r="J111" s="8" t="n"/>
       <c r="K111" s="8" t="n"/>
       <c r="L111" s="8" t="n"/>
+      <c r="M111" s="8" t="n"/>
     </row>
     <row r="112">
       <c r="F112" s="7" t="n"/>
@@ -1716,6 +1852,7 @@
       <c r="J112" s="8" t="n"/>
       <c r="K112" s="8" t="n"/>
       <c r="L112" s="8" t="n"/>
+      <c r="M112" s="8" t="n"/>
     </row>
     <row r="113">
       <c r="F113" s="7" t="n"/>
@@ -1723,6 +1860,7 @@
       <c r="J113" s="8" t="n"/>
       <c r="K113" s="8" t="n"/>
       <c r="L113" s="8" t="n"/>
+      <c r="M113" s="8" t="n"/>
     </row>
     <row r="114">
       <c r="F114" s="7" t="n"/>
@@ -1730,6 +1868,7 @@
       <c r="J114" s="8" t="n"/>
       <c r="K114" s="8" t="n"/>
       <c r="L114" s="8" t="n"/>
+      <c r="M114" s="8" t="n"/>
     </row>
     <row r="115">
       <c r="F115" s="7" t="n"/>
@@ -1737,6 +1876,7 @@
       <c r="J115" s="8" t="n"/>
       <c r="K115" s="8" t="n"/>
       <c r="L115" s="8" t="n"/>
+      <c r="M115" s="8" t="n"/>
     </row>
     <row r="116">
       <c r="F116" s="7" t="n"/>
@@ -1744,6 +1884,7 @@
       <c r="J116" s="8" t="n"/>
       <c r="K116" s="8" t="n"/>
       <c r="L116" s="8" t="n"/>
+      <c r="M116" s="8" t="n"/>
     </row>
     <row r="117">
       <c r="F117" s="7" t="n"/>
@@ -1751,6 +1892,7 @@
       <c r="J117" s="8" t="n"/>
       <c r="K117" s="8" t="n"/>
       <c r="L117" s="8" t="n"/>
+      <c r="M117" s="8" t="n"/>
     </row>
     <row r="118">
       <c r="F118" s="7" t="n"/>
@@ -1758,6 +1900,7 @@
       <c r="J118" s="8" t="n"/>
       <c r="K118" s="8" t="n"/>
       <c r="L118" s="8" t="n"/>
+      <c r="M118" s="8" t="n"/>
     </row>
     <row r="119">
       <c r="F119" s="7" t="n"/>
@@ -1765,6 +1908,7 @@
       <c r="J119" s="8" t="n"/>
       <c r="K119" s="8" t="n"/>
       <c r="L119" s="8" t="n"/>
+      <c r="M119" s="8" t="n"/>
     </row>
     <row r="120">
       <c r="F120" s="7" t="n"/>
@@ -1772,6 +1916,7 @@
       <c r="J120" s="8" t="n"/>
       <c r="K120" s="8" t="n"/>
       <c r="L120" s="8" t="n"/>
+      <c r="M120" s="8" t="n"/>
     </row>
     <row r="121">
       <c r="F121" s="7" t="n"/>
@@ -1779,6 +1924,7 @@
       <c r="J121" s="8" t="n"/>
       <c r="K121" s="8" t="n"/>
       <c r="L121" s="8" t="n"/>
+      <c r="M121" s="8" t="n"/>
     </row>
     <row r="122">
       <c r="F122" s="7" t="n"/>
@@ -1786,6 +1932,7 @@
       <c r="J122" s="8" t="n"/>
       <c r="K122" s="8" t="n"/>
       <c r="L122" s="8" t="n"/>
+      <c r="M122" s="8" t="n"/>
     </row>
     <row r="123">
       <c r="F123" s="7" t="n"/>
@@ -1793,6 +1940,7 @@
       <c r="J123" s="8" t="n"/>
       <c r="K123" s="8" t="n"/>
       <c r="L123" s="8" t="n"/>
+      <c r="M123" s="8" t="n"/>
     </row>
     <row r="124">
       <c r="F124" s="7" t="n"/>
@@ -1800,6 +1948,7 @@
       <c r="J124" s="8" t="n"/>
       <c r="K124" s="8" t="n"/>
       <c r="L124" s="8" t="n"/>
+      <c r="M124" s="8" t="n"/>
     </row>
     <row r="125">
       <c r="F125" s="7" t="n"/>
@@ -1807,6 +1956,7 @@
       <c r="J125" s="8" t="n"/>
       <c r="K125" s="8" t="n"/>
       <c r="L125" s="8" t="n"/>
+      <c r="M125" s="8" t="n"/>
     </row>
     <row r="126">
       <c r="F126" s="7" t="n"/>
@@ -1814,6 +1964,7 @@
       <c r="J126" s="8" t="n"/>
       <c r="K126" s="8" t="n"/>
       <c r="L126" s="8" t="n"/>
+      <c r="M126" s="8" t="n"/>
     </row>
     <row r="127">
       <c r="F127" s="7" t="n"/>
@@ -1821,6 +1972,7 @@
       <c r="J127" s="8" t="n"/>
       <c r="K127" s="8" t="n"/>
       <c r="L127" s="8" t="n"/>
+      <c r="M127" s="8" t="n"/>
     </row>
     <row r="128">
       <c r="F128" s="7" t="n"/>
@@ -1828,6 +1980,7 @@
       <c r="J128" s="8" t="n"/>
       <c r="K128" s="8" t="n"/>
       <c r="L128" s="8" t="n"/>
+      <c r="M128" s="8" t="n"/>
     </row>
     <row r="129">
       <c r="F129" s="7" t="n"/>
@@ -1835,6 +1988,7 @@
       <c r="J129" s="8" t="n"/>
       <c r="K129" s="8" t="n"/>
       <c r="L129" s="8" t="n"/>
+      <c r="M129" s="8" t="n"/>
     </row>
     <row r="130">
       <c r="F130" s="7" t="n"/>
@@ -1842,6 +1996,7 @@
       <c r="J130" s="8" t="n"/>
       <c r="K130" s="8" t="n"/>
       <c r="L130" s="8" t="n"/>
+      <c r="M130" s="8" t="n"/>
     </row>
     <row r="131">
       <c r="F131" s="7" t="n"/>
@@ -1849,6 +2004,7 @@
       <c r="J131" s="8" t="n"/>
       <c r="K131" s="8" t="n"/>
       <c r="L131" s="8" t="n"/>
+      <c r="M131" s="8" t="n"/>
     </row>
     <row r="132">
       <c r="F132" s="7" t="n"/>
@@ -1856,6 +2012,7 @@
       <c r="J132" s="8" t="n"/>
       <c r="K132" s="8" t="n"/>
       <c r="L132" s="8" t="n"/>
+      <c r="M132" s="8" t="n"/>
     </row>
     <row r="133">
       <c r="F133" s="7" t="n"/>
@@ -1863,6 +2020,7 @@
       <c r="J133" s="8" t="n"/>
       <c r="K133" s="8" t="n"/>
       <c r="L133" s="8" t="n"/>
+      <c r="M133" s="8" t="n"/>
     </row>
     <row r="134">
       <c r="F134" s="7" t="n"/>
@@ -1870,6 +2028,7 @@
       <c r="J134" s="8" t="n"/>
       <c r="K134" s="8" t="n"/>
       <c r="L134" s="8" t="n"/>
+      <c r="M134" s="8" t="n"/>
     </row>
     <row r="135">
       <c r="F135" s="7" t="n"/>
@@ -1877,6 +2036,7 @@
       <c r="J135" s="8" t="n"/>
       <c r="K135" s="8" t="n"/>
       <c r="L135" s="8" t="n"/>
+      <c r="M135" s="8" t="n"/>
     </row>
     <row r="136">
       <c r="F136" s="7" t="n"/>
@@ -1884,6 +2044,7 @@
       <c r="J136" s="8" t="n"/>
       <c r="K136" s="8" t="n"/>
       <c r="L136" s="8" t="n"/>
+      <c r="M136" s="8" t="n"/>
     </row>
     <row r="137">
       <c r="F137" s="7" t="n"/>
@@ -1891,6 +2052,7 @@
       <c r="J137" s="8" t="n"/>
       <c r="K137" s="8" t="n"/>
       <c r="L137" s="8" t="n"/>
+      <c r="M137" s="8" t="n"/>
     </row>
     <row r="138">
       <c r="F138" s="7" t="n"/>
@@ -1898,6 +2060,7 @@
       <c r="J138" s="8" t="n"/>
       <c r="K138" s="8" t="n"/>
       <c r="L138" s="8" t="n"/>
+      <c r="M138" s="8" t="n"/>
     </row>
     <row r="139">
       <c r="F139" s="7" t="n"/>
@@ -1905,6 +2068,7 @@
       <c r="J139" s="8" t="n"/>
       <c r="K139" s="8" t="n"/>
       <c r="L139" s="8" t="n"/>
+      <c r="M139" s="8" t="n"/>
     </row>
     <row r="140">
       <c r="F140" s="7" t="n"/>
@@ -1912,6 +2076,7 @@
       <c r="J140" s="8" t="n"/>
       <c r="K140" s="8" t="n"/>
       <c r="L140" s="8" t="n"/>
+      <c r="M140" s="8" t="n"/>
     </row>
     <row r="141">
       <c r="F141" s="7" t="n"/>
@@ -1919,6 +2084,7 @@
       <c r="J141" s="8" t="n"/>
       <c r="K141" s="8" t="n"/>
       <c r="L141" s="8" t="n"/>
+      <c r="M141" s="8" t="n"/>
     </row>
     <row r="142">
       <c r="F142" s="7" t="n"/>
@@ -1926,6 +2092,7 @@
       <c r="J142" s="8" t="n"/>
       <c r="K142" s="8" t="n"/>
       <c r="L142" s="8" t="n"/>
+      <c r="M142" s="8" t="n"/>
     </row>
     <row r="143">
       <c r="F143" s="7" t="n"/>
@@ -1933,6 +2100,7 @@
       <c r="J143" s="8" t="n"/>
       <c r="K143" s="8" t="n"/>
       <c r="L143" s="8" t="n"/>
+      <c r="M143" s="8" t="n"/>
     </row>
     <row r="144">
       <c r="F144" s="7" t="n"/>
@@ -1940,6 +2108,7 @@
       <c r="J144" s="8" t="n"/>
       <c r="K144" s="8" t="n"/>
       <c r="L144" s="8" t="n"/>
+      <c r="M144" s="8" t="n"/>
     </row>
     <row r="145">
       <c r="F145" s="7" t="n"/>
@@ -1947,6 +2116,7 @@
       <c r="J145" s="8" t="n"/>
       <c r="K145" s="8" t="n"/>
       <c r="L145" s="8" t="n"/>
+      <c r="M145" s="8" t="n"/>
     </row>
     <row r="146">
       <c r="F146" s="7" t="n"/>
@@ -1954,6 +2124,7 @@
       <c r="J146" s="8" t="n"/>
       <c r="K146" s="8" t="n"/>
       <c r="L146" s="8" t="n"/>
+      <c r="M146" s="8" t="n"/>
     </row>
     <row r="147">
       <c r="F147" s="7" t="n"/>
@@ -1961,6 +2132,7 @@
       <c r="J147" s="8" t="n"/>
       <c r="K147" s="8" t="n"/>
       <c r="L147" s="8" t="n"/>
+      <c r="M147" s="8" t="n"/>
     </row>
     <row r="148">
       <c r="F148" s="7" t="n"/>
@@ -1968,6 +2140,7 @@
       <c r="J148" s="8" t="n"/>
       <c r="K148" s="8" t="n"/>
       <c r="L148" s="8" t="n"/>
+      <c r="M148" s="8" t="n"/>
     </row>
     <row r="149">
       <c r="F149" s="7" t="n"/>
@@ -1975,6 +2148,7 @@
       <c r="J149" s="8" t="n"/>
       <c r="K149" s="8" t="n"/>
       <c r="L149" s="8" t="n"/>
+      <c r="M149" s="8" t="n"/>
     </row>
     <row r="150">
       <c r="F150" s="7" t="n"/>
@@ -1982,6 +2156,7 @@
       <c r="J150" s="8" t="n"/>
       <c r="K150" s="8" t="n"/>
       <c r="L150" s="8" t="n"/>
+      <c r="M150" s="8" t="n"/>
     </row>
     <row r="151">
       <c r="F151" s="7" t="n"/>
@@ -1989,6 +2164,7 @@
       <c r="J151" s="8" t="n"/>
       <c r="K151" s="8" t="n"/>
       <c r="L151" s="8" t="n"/>
+      <c r="M151" s="8" t="n"/>
     </row>
     <row r="152">
       <c r="F152" s="7" t="n"/>
@@ -1996,6 +2172,7 @@
       <c r="J152" s="8" t="n"/>
       <c r="K152" s="8" t="n"/>
       <c r="L152" s="8" t="n"/>
+      <c r="M152" s="8" t="n"/>
     </row>
     <row r="153">
       <c r="F153" s="7" t="n"/>
@@ -2003,6 +2180,7 @@
       <c r="J153" s="8" t="n"/>
       <c r="K153" s="8" t="n"/>
       <c r="L153" s="8" t="n"/>
+      <c r="M153" s="8" t="n"/>
     </row>
     <row r="154">
       <c r="F154" s="7" t="n"/>
@@ -2010,6 +2188,7 @@
       <c r="J154" s="8" t="n"/>
       <c r="K154" s="8" t="n"/>
       <c r="L154" s="8" t="n"/>
+      <c r="M154" s="8" t="n"/>
     </row>
     <row r="155">
       <c r="F155" s="7" t="n"/>
@@ -2017,6 +2196,7 @@
       <c r="J155" s="8" t="n"/>
       <c r="K155" s="8" t="n"/>
       <c r="L155" s="8" t="n"/>
+      <c r="M155" s="8" t="n"/>
     </row>
     <row r="156">
       <c r="F156" s="7" t="n"/>
@@ -2024,6 +2204,7 @@
       <c r="J156" s="8" t="n"/>
       <c r="K156" s="8" t="n"/>
       <c r="L156" s="8" t="n"/>
+      <c r="M156" s="8" t="n"/>
     </row>
     <row r="157">
       <c r="F157" s="7" t="n"/>
@@ -2031,6 +2212,7 @@
       <c r="J157" s="8" t="n"/>
       <c r="K157" s="8" t="n"/>
       <c r="L157" s="8" t="n"/>
+      <c r="M157" s="8" t="n"/>
     </row>
     <row r="158">
       <c r="F158" s="7" t="n"/>
@@ -2038,6 +2220,7 @@
       <c r="J158" s="8" t="n"/>
       <c r="K158" s="8" t="n"/>
       <c r="L158" s="8" t="n"/>
+      <c r="M158" s="8" t="n"/>
     </row>
     <row r="159">
       <c r="F159" s="7" t="n"/>
@@ -2045,6 +2228,7 @@
       <c r="J159" s="8" t="n"/>
       <c r="K159" s="8" t="n"/>
       <c r="L159" s="8" t="n"/>
+      <c r="M159" s="8" t="n"/>
     </row>
     <row r="160">
       <c r="F160" s="7" t="n"/>
@@ -2052,6 +2236,7 @@
       <c r="J160" s="8" t="n"/>
       <c r="K160" s="8" t="n"/>
       <c r="L160" s="8" t="n"/>
+      <c r="M160" s="8" t="n"/>
     </row>
     <row r="161">
       <c r="F161" s="7" t="n"/>
@@ -2059,6 +2244,7 @@
       <c r="J161" s="8" t="n"/>
       <c r="K161" s="8" t="n"/>
       <c r="L161" s="8" t="n"/>
+      <c r="M161" s="8" t="n"/>
     </row>
     <row r="162">
       <c r="F162" s="7" t="n"/>
@@ -2066,6 +2252,7 @@
       <c r="J162" s="8" t="n"/>
       <c r="K162" s="8" t="n"/>
       <c r="L162" s="8" t="n"/>
+      <c r="M162" s="8" t="n"/>
     </row>
     <row r="163">
       <c r="F163" s="7" t="n"/>
@@ -2073,6 +2260,7 @@
       <c r="J163" s="8" t="n"/>
       <c r="K163" s="8" t="n"/>
       <c r="L163" s="8" t="n"/>
+      <c r="M163" s="8" t="n"/>
     </row>
     <row r="164">
       <c r="F164" s="7" t="n"/>
@@ -2080,6 +2268,7 @@
       <c r="J164" s="8" t="n"/>
       <c r="K164" s="8" t="n"/>
       <c r="L164" s="8" t="n"/>
+      <c r="M164" s="8" t="n"/>
     </row>
     <row r="165">
       <c r="F165" s="7" t="n"/>
@@ -2087,6 +2276,7 @@
       <c r="J165" s="8" t="n"/>
       <c r="K165" s="8" t="n"/>
       <c r="L165" s="8" t="n"/>
+      <c r="M165" s="8" t="n"/>
     </row>
     <row r="166">
       <c r="F166" s="7" t="n"/>
@@ -2094,6 +2284,7 @@
       <c r="J166" s="8" t="n"/>
       <c r="K166" s="8" t="n"/>
       <c r="L166" s="8" t="n"/>
+      <c r="M166" s="8" t="n"/>
     </row>
     <row r="167">
       <c r="F167" s="7" t="n"/>
@@ -2101,6 +2292,7 @@
       <c r="J167" s="8" t="n"/>
       <c r="K167" s="8" t="n"/>
       <c r="L167" s="8" t="n"/>
+      <c r="M167" s="8" t="n"/>
     </row>
     <row r="168">
       <c r="F168" s="7" t="n"/>
@@ -2108,6 +2300,7 @@
       <c r="J168" s="8" t="n"/>
       <c r="K168" s="8" t="n"/>
       <c r="L168" s="8" t="n"/>
+      <c r="M168" s="8" t="n"/>
     </row>
     <row r="169">
       <c r="F169" s="7" t="n"/>
@@ -2115,6 +2308,7 @@
       <c r="J169" s="8" t="n"/>
       <c r="K169" s="8" t="n"/>
       <c r="L169" s="8" t="n"/>
+      <c r="M169" s="8" t="n"/>
     </row>
     <row r="170">
       <c r="F170" s="7" t="n"/>
@@ -2122,6 +2316,7 @@
       <c r="J170" s="8" t="n"/>
       <c r="K170" s="8" t="n"/>
       <c r="L170" s="8" t="n"/>
+      <c r="M170" s="8" t="n"/>
     </row>
     <row r="171">
       <c r="F171" s="7" t="n"/>
@@ -2129,6 +2324,7 @@
       <c r="J171" s="8" t="n"/>
       <c r="K171" s="8" t="n"/>
       <c r="L171" s="8" t="n"/>
+      <c r="M171" s="8" t="n"/>
     </row>
     <row r="172">
       <c r="F172" s="7" t="n"/>
@@ -2136,6 +2332,7 @@
       <c r="J172" s="8" t="n"/>
       <c r="K172" s="8" t="n"/>
       <c r="L172" s="8" t="n"/>
+      <c r="M172" s="8" t="n"/>
     </row>
     <row r="173">
       <c r="F173" s="7" t="n"/>
@@ -2143,6 +2340,7 @@
       <c r="J173" s="8" t="n"/>
       <c r="K173" s="8" t="n"/>
       <c r="L173" s="8" t="n"/>
+      <c r="M173" s="8" t="n"/>
     </row>
     <row r="174">
       <c r="F174" s="7" t="n"/>
@@ -2150,6 +2348,7 @@
       <c r="J174" s="8" t="n"/>
       <c r="K174" s="8" t="n"/>
       <c r="L174" s="8" t="n"/>
+      <c r="M174" s="8" t="n"/>
     </row>
     <row r="175">
       <c r="F175" s="7" t="n"/>
@@ -2157,6 +2356,7 @@
       <c r="J175" s="8" t="n"/>
       <c r="K175" s="8" t="n"/>
       <c r="L175" s="8" t="n"/>
+      <c r="M175" s="8" t="n"/>
     </row>
     <row r="176">
       <c r="F176" s="7" t="n"/>
@@ -2164,6 +2364,7 @@
       <c r="J176" s="8" t="n"/>
       <c r="K176" s="8" t="n"/>
       <c r="L176" s="8" t="n"/>
+      <c r="M176" s="8" t="n"/>
     </row>
     <row r="177">
       <c r="F177" s="7" t="n"/>
@@ -2171,6 +2372,7 @@
       <c r="J177" s="8" t="n"/>
       <c r="K177" s="8" t="n"/>
       <c r="L177" s="8" t="n"/>
+      <c r="M177" s="8" t="n"/>
     </row>
     <row r="178">
       <c r="F178" s="7" t="n"/>
@@ -2178,6 +2380,7 @@
       <c r="J178" s="8" t="n"/>
       <c r="K178" s="8" t="n"/>
       <c r="L178" s="8" t="n"/>
+      <c r="M178" s="8" t="n"/>
     </row>
     <row r="179">
       <c r="F179" s="7" t="n"/>
@@ -2185,6 +2388,7 @@
       <c r="J179" s="8" t="n"/>
       <c r="K179" s="8" t="n"/>
       <c r="L179" s="8" t="n"/>
+      <c r="M179" s="8" t="n"/>
     </row>
     <row r="180">
       <c r="F180" s="7" t="n"/>
@@ -2192,6 +2396,7 @@
       <c r="J180" s="8" t="n"/>
       <c r="K180" s="8" t="n"/>
       <c r="L180" s="8" t="n"/>
+      <c r="M180" s="8" t="n"/>
     </row>
     <row r="181">
       <c r="F181" s="7" t="n"/>
@@ -2199,6 +2404,7 @@
       <c r="J181" s="8" t="n"/>
       <c r="K181" s="8" t="n"/>
       <c r="L181" s="8" t="n"/>
+      <c r="M181" s="8" t="n"/>
     </row>
     <row r="182">
       <c r="F182" s="7" t="n"/>
@@ -2206,6 +2412,7 @@
       <c r="J182" s="8" t="n"/>
       <c r="K182" s="8" t="n"/>
       <c r="L182" s="8" t="n"/>
+      <c r="M182" s="8" t="n"/>
     </row>
     <row r="183">
       <c r="F183" s="7" t="n"/>
@@ -2213,6 +2420,7 @@
       <c r="J183" s="8" t="n"/>
       <c r="K183" s="8" t="n"/>
       <c r="L183" s="8" t="n"/>
+      <c r="M183" s="8" t="n"/>
     </row>
     <row r="184">
       <c r="F184" s="7" t="n"/>
@@ -2220,6 +2428,7 @@
       <c r="J184" s="8" t="n"/>
       <c r="K184" s="8" t="n"/>
       <c r="L184" s="8" t="n"/>
+      <c r="M184" s="8" t="n"/>
     </row>
     <row r="185">
       <c r="F185" s="7" t="n"/>
@@ -2227,6 +2436,7 @@
       <c r="J185" s="8" t="n"/>
       <c r="K185" s="8" t="n"/>
       <c r="L185" s="8" t="n"/>
+      <c r="M185" s="8" t="n"/>
     </row>
     <row r="186">
       <c r="F186" s="7" t="n"/>
@@ -2234,6 +2444,7 @@
       <c r="J186" s="8" t="n"/>
       <c r="K186" s="8" t="n"/>
       <c r="L186" s="8" t="n"/>
+      <c r="M186" s="8" t="n"/>
     </row>
     <row r="187">
       <c r="F187" s="7" t="n"/>
@@ -2241,6 +2452,7 @@
       <c r="J187" s="8" t="n"/>
       <c r="K187" s="8" t="n"/>
       <c r="L187" s="8" t="n"/>
+      <c r="M187" s="8" t="n"/>
     </row>
     <row r="188">
       <c r="F188" s="7" t="n"/>
@@ -2248,6 +2460,7 @@
       <c r="J188" s="8" t="n"/>
       <c r="K188" s="8" t="n"/>
       <c r="L188" s="8" t="n"/>
+      <c r="M188" s="8" t="n"/>
     </row>
     <row r="189">
       <c r="F189" s="7" t="n"/>
@@ -2255,6 +2468,7 @@
       <c r="J189" s="8" t="n"/>
       <c r="K189" s="8" t="n"/>
       <c r="L189" s="8" t="n"/>
+      <c r="M189" s="8" t="n"/>
     </row>
     <row r="190">
       <c r="F190" s="7" t="n"/>
@@ -2262,6 +2476,7 @@
       <c r="J190" s="8" t="n"/>
       <c r="K190" s="8" t="n"/>
       <c r="L190" s="8" t="n"/>
+      <c r="M190" s="8" t="n"/>
     </row>
     <row r="191">
       <c r="F191" s="7" t="n"/>
@@ -2269,6 +2484,7 @@
       <c r="J191" s="8" t="n"/>
       <c r="K191" s="8" t="n"/>
       <c r="L191" s="8" t="n"/>
+      <c r="M191" s="8" t="n"/>
     </row>
     <row r="192">
       <c r="F192" s="7" t="n"/>
@@ -2276,6 +2492,7 @@
       <c r="J192" s="8" t="n"/>
       <c r="K192" s="8" t="n"/>
       <c r="L192" s="8" t="n"/>
+      <c r="M192" s="8" t="n"/>
     </row>
     <row r="193">
       <c r="F193" s="7" t="n"/>
@@ -2283,6 +2500,7 @@
       <c r="J193" s="8" t="n"/>
       <c r="K193" s="8" t="n"/>
       <c r="L193" s="8" t="n"/>
+      <c r="M193" s="8" t="n"/>
     </row>
     <row r="194">
       <c r="F194" s="7" t="n"/>
@@ -2290,6 +2508,7 @@
       <c r="J194" s="8" t="n"/>
       <c r="K194" s="8" t="n"/>
       <c r="L194" s="8" t="n"/>
+      <c r="M194" s="8" t="n"/>
     </row>
     <row r="195">
       <c r="F195" s="7" t="n"/>
@@ -2297,6 +2516,7 @@
       <c r="J195" s="8" t="n"/>
       <c r="K195" s="8" t="n"/>
       <c r="L195" s="8" t="n"/>
+      <c r="M195" s="8" t="n"/>
     </row>
     <row r="196">
       <c r="F196" s="7" t="n"/>
@@ -2304,6 +2524,7 @@
       <c r="J196" s="8" t="n"/>
       <c r="K196" s="8" t="n"/>
       <c r="L196" s="8" t="n"/>
+      <c r="M196" s="8" t="n"/>
     </row>
     <row r="197">
       <c r="F197" s="7" t="n"/>
@@ -2311,6 +2532,7 @@
       <c r="J197" s="8" t="n"/>
       <c r="K197" s="8" t="n"/>
       <c r="L197" s="8" t="n"/>
+      <c r="M197" s="8" t="n"/>
     </row>
     <row r="198">
       <c r="F198" s="7" t="n"/>
@@ -2318,6 +2540,7 @@
       <c r="J198" s="8" t="n"/>
       <c r="K198" s="8" t="n"/>
       <c r="L198" s="8" t="n"/>
+      <c r="M198" s="8" t="n"/>
     </row>
     <row r="199">
       <c r="F199" s="7" t="n"/>
@@ -2325,6 +2548,7 @@
       <c r="J199" s="8" t="n"/>
       <c r="K199" s="8" t="n"/>
       <c r="L199" s="8" t="n"/>
+      <c r="M199" s="8" t="n"/>
     </row>
     <row r="200">
       <c r="F200" s="7" t="n"/>
@@ -2332,6 +2556,7 @@
       <c r="J200" s="8" t="n"/>
       <c r="K200" s="8" t="n"/>
       <c r="L200" s="8" t="n"/>
+      <c r="M200" s="8" t="n"/>
     </row>
     <row r="201">
       <c r="F201" s="7" t="n"/>
@@ -2339,6 +2564,7 @@
       <c r="J201" s="8" t="n"/>
       <c r="K201" s="8" t="n"/>
       <c r="L201" s="8" t="n"/>
+      <c r="M201" s="8" t="n"/>
     </row>
     <row r="202">
       <c r="F202" s="7" t="n"/>
@@ -2346,6 +2572,7 @@
       <c r="J202" s="8" t="n"/>
       <c r="K202" s="8" t="n"/>
       <c r="L202" s="8" t="n"/>
+      <c r="M202" s="8" t="n"/>
     </row>
     <row r="203">
       <c r="F203" s="7" t="n"/>
@@ -2353,6 +2580,7 @@
       <c r="J203" s="8" t="n"/>
       <c r="K203" s="8" t="n"/>
       <c r="L203" s="8" t="n"/>
+      <c r="M203" s="8" t="n"/>
     </row>
     <row r="204">
       <c r="F204" s="7" t="n"/>
@@ -2360,6 +2588,7 @@
       <c r="J204" s="8" t="n"/>
       <c r="K204" s="8" t="n"/>
       <c r="L204" s="8" t="n"/>
+      <c r="M204" s="8" t="n"/>
     </row>
     <row r="205">
       <c r="F205" s="7" t="n"/>
@@ -2367,6 +2596,7 @@
       <c r="J205" s="8" t="n"/>
       <c r="K205" s="8" t="n"/>
       <c r="L205" s="8" t="n"/>
+      <c r="M205" s="8" t="n"/>
     </row>
     <row r="206">
       <c r="F206" s="7" t="n"/>
@@ -2374,6 +2604,7 @@
       <c r="J206" s="8" t="n"/>
       <c r="K206" s="8" t="n"/>
       <c r="L206" s="8" t="n"/>
+      <c r="M206" s="8" t="n"/>
     </row>
     <row r="207">
       <c r="F207" s="7" t="n"/>
@@ -2381,6 +2612,7 @@
       <c r="J207" s="8" t="n"/>
       <c r="K207" s="8" t="n"/>
       <c r="L207" s="8" t="n"/>
+      <c r="M207" s="8" t="n"/>
     </row>
     <row r="208">
       <c r="F208" s="7" t="n"/>
@@ -2388,6 +2620,7 @@
       <c r="J208" s="8" t="n"/>
       <c r="K208" s="8" t="n"/>
       <c r="L208" s="8" t="n"/>
+      <c r="M208" s="8" t="n"/>
     </row>
     <row r="209">
       <c r="F209" s="7" t="n"/>
@@ -2395,6 +2628,7 @@
       <c r="J209" s="8" t="n"/>
       <c r="K209" s="8" t="n"/>
       <c r="L209" s="8" t="n"/>
+      <c r="M209" s="8" t="n"/>
     </row>
     <row r="210">
       <c r="F210" s="7" t="n"/>
@@ -2402,6 +2636,7 @@
       <c r="J210" s="8" t="n"/>
       <c r="K210" s="8" t="n"/>
       <c r="L210" s="8" t="n"/>
+      <c r="M210" s="8" t="n"/>
     </row>
     <row r="211">
       <c r="F211" s="7" t="n"/>
@@ -2409,6 +2644,7 @@
       <c r="J211" s="8" t="n"/>
       <c r="K211" s="8" t="n"/>
       <c r="L211" s="8" t="n"/>
+      <c r="M211" s="8" t="n"/>
     </row>
     <row r="212">
       <c r="F212" s="7" t="n"/>
@@ -2416,6 +2652,7 @@
       <c r="J212" s="8" t="n"/>
       <c r="K212" s="8" t="n"/>
       <c r="L212" s="8" t="n"/>
+      <c r="M212" s="8" t="n"/>
     </row>
     <row r="213">
       <c r="F213" s="7" t="n"/>
@@ -2423,6 +2660,7 @@
       <c r="J213" s="8" t="n"/>
       <c r="K213" s="8" t="n"/>
       <c r="L213" s="8" t="n"/>
+      <c r="M213" s="8" t="n"/>
     </row>
     <row r="214">
       <c r="F214" s="7" t="n"/>
@@ -2430,6 +2668,7 @@
       <c r="J214" s="8" t="n"/>
       <c r="K214" s="8" t="n"/>
       <c r="L214" s="8" t="n"/>
+      <c r="M214" s="8" t="n"/>
     </row>
     <row r="215">
       <c r="F215" s="7" t="n"/>
@@ -2437,6 +2676,7 @@
       <c r="J215" s="8" t="n"/>
       <c r="K215" s="8" t="n"/>
       <c r="L215" s="8" t="n"/>
+      <c r="M215" s="8" t="n"/>
     </row>
     <row r="216">
       <c r="F216" s="7" t="n"/>
@@ -2444,6 +2684,7 @@
       <c r="J216" s="8" t="n"/>
       <c r="K216" s="8" t="n"/>
       <c r="L216" s="8" t="n"/>
+      <c r="M216" s="8" t="n"/>
     </row>
     <row r="217">
       <c r="F217" s="7" t="n"/>
@@ -2451,6 +2692,7 @@
       <c r="J217" s="8" t="n"/>
       <c r="K217" s="8" t="n"/>
       <c r="L217" s="8" t="n"/>
+      <c r="M217" s="8" t="n"/>
     </row>
     <row r="218">
       <c r="F218" s="7" t="n"/>
@@ -2458,6 +2700,7 @@
       <c r="J218" s="8" t="n"/>
       <c r="K218" s="8" t="n"/>
       <c r="L218" s="8" t="n"/>
+      <c r="M218" s="8" t="n"/>
     </row>
     <row r="219">
       <c r="F219" s="7" t="n"/>
@@ -2465,6 +2708,7 @@
       <c r="J219" s="8" t="n"/>
       <c r="K219" s="8" t="n"/>
       <c r="L219" s="8" t="n"/>
+      <c r="M219" s="8" t="n"/>
     </row>
     <row r="220">
       <c r="F220" s="7" t="n"/>
@@ -2472,6 +2716,7 @@
       <c r="J220" s="8" t="n"/>
       <c r="K220" s="8" t="n"/>
       <c r="L220" s="8" t="n"/>
+      <c r="M220" s="8" t="n"/>
     </row>
     <row r="221">
       <c r="F221" s="7" t="n"/>
@@ -2479,6 +2724,7 @@
       <c r="J221" s="8" t="n"/>
       <c r="K221" s="8" t="n"/>
       <c r="L221" s="8" t="n"/>
+      <c r="M221" s="8" t="n"/>
     </row>
     <row r="222">
       <c r="F222" s="7" t="n"/>
@@ -2486,6 +2732,7 @@
       <c r="J222" s="8" t="n"/>
       <c r="K222" s="8" t="n"/>
       <c r="L222" s="8" t="n"/>
+      <c r="M222" s="8" t="n"/>
     </row>
     <row r="223">
       <c r="F223" s="7" t="n"/>
@@ -2493,6 +2740,7 @@
       <c r="J223" s="8" t="n"/>
       <c r="K223" s="8" t="n"/>
       <c r="L223" s="8" t="n"/>
+      <c r="M223" s="8" t="n"/>
     </row>
     <row r="224">
       <c r="F224" s="7" t="n"/>
@@ -2500,6 +2748,7 @@
       <c r="J224" s="8" t="n"/>
       <c r="K224" s="8" t="n"/>
       <c r="L224" s="8" t="n"/>
+      <c r="M224" s="8" t="n"/>
     </row>
     <row r="225">
       <c r="F225" s="7" t="n"/>
@@ -2507,6 +2756,7 @@
       <c r="J225" s="8" t="n"/>
       <c r="K225" s="8" t="n"/>
       <c r="L225" s="8" t="n"/>
+      <c r="M225" s="8" t="n"/>
     </row>
     <row r="226">
       <c r="F226" s="7" t="n"/>
@@ -2514,6 +2764,7 @@
       <c r="J226" s="8" t="n"/>
       <c r="K226" s="8" t="n"/>
       <c r="L226" s="8" t="n"/>
+      <c r="M226" s="8" t="n"/>
     </row>
     <row r="227">
       <c r="F227" s="7" t="n"/>
@@ -2521,6 +2772,7 @@
       <c r="J227" s="8" t="n"/>
       <c r="K227" s="8" t="n"/>
       <c r="L227" s="8" t="n"/>
+      <c r="M227" s="8" t="n"/>
     </row>
     <row r="228">
       <c r="F228" s="7" t="n"/>
@@ -2528,6 +2780,7 @@
       <c r="J228" s="8" t="n"/>
       <c r="K228" s="8" t="n"/>
       <c r="L228" s="8" t="n"/>
+      <c r="M228" s="8" t="n"/>
     </row>
     <row r="229">
       <c r="F229" s="7" t="n"/>
@@ -2535,6 +2788,7 @@
       <c r="J229" s="8" t="n"/>
       <c r="K229" s="8" t="n"/>
       <c r="L229" s="8" t="n"/>
+      <c r="M229" s="8" t="n"/>
     </row>
     <row r="230">
       <c r="F230" s="7" t="n"/>
@@ -2542,6 +2796,7 @@
       <c r="J230" s="8" t="n"/>
       <c r="K230" s="8" t="n"/>
       <c r="L230" s="8" t="n"/>
+      <c r="M230" s="8" t="n"/>
     </row>
     <row r="231">
       <c r="F231" s="7" t="n"/>
@@ -2549,6 +2804,7 @@
       <c r="J231" s="8" t="n"/>
       <c r="K231" s="8" t="n"/>
       <c r="L231" s="8" t="n"/>
+      <c r="M231" s="8" t="n"/>
     </row>
     <row r="232">
       <c r="F232" s="7" t="n"/>
@@ -2556,6 +2812,7 @@
       <c r="J232" s="8" t="n"/>
       <c r="K232" s="8" t="n"/>
       <c r="L232" s="8" t="n"/>
+      <c r="M232" s="8" t="n"/>
     </row>
     <row r="233">
       <c r="F233" s="7" t="n"/>
@@ -2563,6 +2820,7 @@
       <c r="J233" s="8" t="n"/>
       <c r="K233" s="8" t="n"/>
       <c r="L233" s="8" t="n"/>
+      <c r="M233" s="8" t="n"/>
     </row>
     <row r="234">
       <c r="F234" s="7" t="n"/>
@@ -2570,6 +2828,7 @@
       <c r="J234" s="8" t="n"/>
       <c r="K234" s="8" t="n"/>
       <c r="L234" s="8" t="n"/>
+      <c r="M234" s="8" t="n"/>
     </row>
     <row r="235">
       <c r="F235" s="7" t="n"/>
@@ -2577,6 +2836,7 @@
       <c r="J235" s="8" t="n"/>
       <c r="K235" s="8" t="n"/>
       <c r="L235" s="8" t="n"/>
+      <c r="M235" s="8" t="n"/>
     </row>
     <row r="236">
       <c r="F236" s="7" t="n"/>
@@ -2584,6 +2844,7 @@
       <c r="J236" s="8" t="n"/>
       <c r="K236" s="8" t="n"/>
       <c r="L236" s="8" t="n"/>
+      <c r="M236" s="8" t="n"/>
     </row>
     <row r="237">
       <c r="F237" s="7" t="n"/>
@@ -2591,6 +2852,7 @@
       <c r="J237" s="8" t="n"/>
       <c r="K237" s="8" t="n"/>
       <c r="L237" s="8" t="n"/>
+      <c r="M237" s="8" t="n"/>
     </row>
     <row r="238">
       <c r="F238" s="7" t="n"/>
@@ -2598,6 +2860,7 @@
       <c r="J238" s="8" t="n"/>
       <c r="K238" s="8" t="n"/>
       <c r="L238" s="8" t="n"/>
+      <c r="M238" s="8" t="n"/>
     </row>
     <row r="239">
       <c r="F239" s="7" t="n"/>
@@ -2605,6 +2868,7 @@
       <c r="J239" s="8" t="n"/>
       <c r="K239" s="8" t="n"/>
       <c r="L239" s="8" t="n"/>
+      <c r="M239" s="8" t="n"/>
     </row>
     <row r="240">
       <c r="F240" s="7" t="n"/>
@@ -2612,6 +2876,7 @@
       <c r="J240" s="8" t="n"/>
       <c r="K240" s="8" t="n"/>
       <c r="L240" s="8" t="n"/>
+      <c r="M240" s="8" t="n"/>
     </row>
     <row r="241">
       <c r="F241" s="7" t="n"/>
@@ -2619,6 +2884,7 @@
       <c r="J241" s="8" t="n"/>
       <c r="K241" s="8" t="n"/>
       <c r="L241" s="8" t="n"/>
+      <c r="M241" s="8" t="n"/>
     </row>
     <row r="242">
       <c r="F242" s="7" t="n"/>
@@ -2626,6 +2892,7 @@
       <c r="J242" s="8" t="n"/>
       <c r="K242" s="8" t="n"/>
       <c r="L242" s="8" t="n"/>
+      <c r="M242" s="8" t="n"/>
     </row>
     <row r="243">
       <c r="F243" s="7" t="n"/>
@@ -2633,6 +2900,7 @@
       <c r="J243" s="8" t="n"/>
       <c r="K243" s="8" t="n"/>
       <c r="L243" s="8" t="n"/>
+      <c r="M243" s="8" t="n"/>
     </row>
     <row r="244">
       <c r="F244" s="7" t="n"/>
@@ -2640,6 +2908,7 @@
       <c r="J244" s="8" t="n"/>
       <c r="K244" s="8" t="n"/>
       <c r="L244" s="8" t="n"/>
+      <c r="M244" s="8" t="n"/>
     </row>
     <row r="245">
       <c r="F245" s="7" t="n"/>
@@ -2647,6 +2916,7 @@
       <c r="J245" s="8" t="n"/>
       <c r="K245" s="8" t="n"/>
       <c r="L245" s="8" t="n"/>
+      <c r="M245" s="8" t="n"/>
     </row>
     <row r="246">
       <c r="F246" s="7" t="n"/>
@@ -2654,6 +2924,7 @@
       <c r="J246" s="8" t="n"/>
       <c r="K246" s="8" t="n"/>
       <c r="L246" s="8" t="n"/>
+      <c r="M246" s="8" t="n"/>
     </row>
     <row r="247">
       <c r="F247" s="7" t="n"/>
@@ -2661,6 +2932,7 @@
       <c r="J247" s="8" t="n"/>
       <c r="K247" s="8" t="n"/>
       <c r="L247" s="8" t="n"/>
+      <c r="M247" s="8" t="n"/>
     </row>
     <row r="248">
       <c r="F248" s="7" t="n"/>
@@ -2668,6 +2940,7 @@
       <c r="J248" s="8" t="n"/>
       <c r="K248" s="8" t="n"/>
       <c r="L248" s="8" t="n"/>
+      <c r="M248" s="8" t="n"/>
     </row>
     <row r="249">
       <c r="F249" s="7" t="n"/>
@@ -2675,6 +2948,7 @@
       <c r="J249" s="8" t="n"/>
       <c r="K249" s="8" t="n"/>
       <c r="L249" s="8" t="n"/>
+      <c r="M249" s="8" t="n"/>
     </row>
     <row r="250">
       <c r="F250" s="7" t="n"/>
@@ -2682,6 +2956,7 @@
       <c r="J250" s="8" t="n"/>
       <c r="K250" s="8" t="n"/>
       <c r="L250" s="8" t="n"/>
+      <c r="M250" s="8" t="n"/>
     </row>
     <row r="251">
       <c r="F251" s="7" t="n"/>
@@ -2689,6 +2964,7 @@
       <c r="J251" s="8" t="n"/>
       <c r="K251" s="8" t="n"/>
       <c r="L251" s="8" t="n"/>
+      <c r="M251" s="8" t="n"/>
     </row>
     <row r="252">
       <c r="F252" s="7" t="n"/>
@@ -2696,6 +2972,7 @@
       <c r="J252" s="8" t="n"/>
       <c r="K252" s="8" t="n"/>
       <c r="L252" s="8" t="n"/>
+      <c r="M252" s="8" t="n"/>
     </row>
     <row r="253">
       <c r="F253" s="7" t="n"/>
@@ -2703,6 +2980,7 @@
       <c r="J253" s="8" t="n"/>
       <c r="K253" s="8" t="n"/>
       <c r="L253" s="8" t="n"/>
+      <c r="M253" s="8" t="n"/>
     </row>
     <row r="254">
       <c r="F254" s="7" t="n"/>
@@ -2710,6 +2988,7 @@
       <c r="J254" s="8" t="n"/>
       <c r="K254" s="8" t="n"/>
       <c r="L254" s="8" t="n"/>
+      <c r="M254" s="8" t="n"/>
     </row>
     <row r="255">
       <c r="F255" s="7" t="n"/>
@@ -2717,6 +2996,7 @@
       <c r="J255" s="8" t="n"/>
       <c r="K255" s="8" t="n"/>
       <c r="L255" s="8" t="n"/>
+      <c r="M255" s="8" t="n"/>
     </row>
     <row r="256">
       <c r="F256" s="7" t="n"/>
@@ -2724,6 +3004,7 @@
       <c r="J256" s="8" t="n"/>
       <c r="K256" s="8" t="n"/>
       <c r="L256" s="8" t="n"/>
+      <c r="M256" s="8" t="n"/>
     </row>
     <row r="257">
       <c r="F257" s="7" t="n"/>
@@ -2731,6 +3012,7 @@
       <c r="J257" s="8" t="n"/>
       <c r="K257" s="8" t="n"/>
       <c r="L257" s="8" t="n"/>
+      <c r="M257" s="8" t="n"/>
     </row>
     <row r="258">
       <c r="F258" s="7" t="n"/>
@@ -2738,6 +3020,7 @@
       <c r="J258" s="8" t="n"/>
       <c r="K258" s="8" t="n"/>
       <c r="L258" s="8" t="n"/>
+      <c r="M258" s="8" t="n"/>
     </row>
     <row r="259">
       <c r="F259" s="7" t="n"/>
@@ -2745,6 +3028,7 @@
       <c r="J259" s="8" t="n"/>
       <c r="K259" s="8" t="n"/>
       <c r="L259" s="8" t="n"/>
+      <c r="M259" s="8" t="n"/>
     </row>
     <row r="260">
       <c r="F260" s="7" t="n"/>
@@ -2752,6 +3036,7 @@
       <c r="J260" s="8" t="n"/>
       <c r="K260" s="8" t="n"/>
       <c r="L260" s="8" t="n"/>
+      <c r="M260" s="8" t="n"/>
     </row>
     <row r="261">
       <c r="F261" s="7" t="n"/>
@@ -2759,6 +3044,7 @@
       <c r="J261" s="8" t="n"/>
       <c r="K261" s="8" t="n"/>
       <c r="L261" s="8" t="n"/>
+      <c r="M261" s="8" t="n"/>
     </row>
     <row r="262">
       <c r="F262" s="7" t="n"/>
@@ -2766,6 +3052,7 @@
       <c r="J262" s="8" t="n"/>
       <c r="K262" s="8" t="n"/>
       <c r="L262" s="8" t="n"/>
+      <c r="M262" s="8" t="n"/>
     </row>
     <row r="263">
       <c r="F263" s="7" t="n"/>
@@ -2773,6 +3060,7 @@
       <c r="J263" s="8" t="n"/>
       <c r="K263" s="8" t="n"/>
       <c r="L263" s="8" t="n"/>
+      <c r="M263" s="8" t="n"/>
     </row>
     <row r="264">
       <c r="F264" s="7" t="n"/>
@@ -2780,6 +3068,7 @@
       <c r="J264" s="8" t="n"/>
       <c r="K264" s="8" t="n"/>
       <c r="L264" s="8" t="n"/>
+      <c r="M264" s="8" t="n"/>
     </row>
     <row r="265">
       <c r="F265" s="7" t="n"/>
@@ -2787,6 +3076,7 @@
       <c r="J265" s="8" t="n"/>
       <c r="K265" s="8" t="n"/>
       <c r="L265" s="8" t="n"/>
+      <c r="M265" s="8" t="n"/>
     </row>
     <row r="266">
       <c r="F266" s="7" t="n"/>
@@ -2794,6 +3084,7 @@
       <c r="J266" s="8" t="n"/>
       <c r="K266" s="8" t="n"/>
       <c r="L266" s="8" t="n"/>
+      <c r="M266" s="8" t="n"/>
     </row>
     <row r="267">
       <c r="F267" s="7" t="n"/>
@@ -2801,6 +3092,7 @@
       <c r="J267" s="8" t="n"/>
       <c r="K267" s="8" t="n"/>
       <c r="L267" s="8" t="n"/>
+      <c r="M267" s="8" t="n"/>
     </row>
     <row r="268">
       <c r="F268" s="7" t="n"/>
@@ -2808,6 +3100,7 @@
       <c r="J268" s="8" t="n"/>
       <c r="K268" s="8" t="n"/>
       <c r="L268" s="8" t="n"/>
+      <c r="M268" s="8" t="n"/>
     </row>
     <row r="269">
       <c r="F269" s="7" t="n"/>
@@ -2815,6 +3108,7 @@
       <c r="J269" s="8" t="n"/>
       <c r="K269" s="8" t="n"/>
       <c r="L269" s="8" t="n"/>
+      <c r="M269" s="8" t="n"/>
     </row>
     <row r="270">
       <c r="F270" s="7" t="n"/>
@@ -2822,6 +3116,7 @@
       <c r="J270" s="8" t="n"/>
       <c r="K270" s="8" t="n"/>
       <c r="L270" s="8" t="n"/>
+      <c r="M270" s="8" t="n"/>
     </row>
     <row r="271">
       <c r="F271" s="7" t="n"/>
@@ -2829,6 +3124,7 @@
       <c r="J271" s="8" t="n"/>
       <c r="K271" s="8" t="n"/>
       <c r="L271" s="8" t="n"/>
+      <c r="M271" s="8" t="n"/>
     </row>
     <row r="272">
       <c r="F272" s="7" t="n"/>
@@ -2836,6 +3132,7 @@
       <c r="J272" s="8" t="n"/>
       <c r="K272" s="8" t="n"/>
       <c r="L272" s="8" t="n"/>
+      <c r="M272" s="8" t="n"/>
     </row>
     <row r="273">
       <c r="F273" s="7" t="n"/>
@@ -2843,6 +3140,7 @@
       <c r="J273" s="8" t="n"/>
       <c r="K273" s="8" t="n"/>
       <c r="L273" s="8" t="n"/>
+      <c r="M273" s="8" t="n"/>
     </row>
     <row r="274">
       <c r="F274" s="7" t="n"/>
@@ -2850,6 +3148,7 @@
       <c r="J274" s="8" t="n"/>
       <c r="K274" s="8" t="n"/>
       <c r="L274" s="8" t="n"/>
+      <c r="M274" s="8" t="n"/>
     </row>
     <row r="275">
       <c r="F275" s="7" t="n"/>
@@ -2857,6 +3156,7 @@
       <c r="J275" s="8" t="n"/>
       <c r="K275" s="8" t="n"/>
       <c r="L275" s="8" t="n"/>
+      <c r="M275" s="8" t="n"/>
     </row>
     <row r="276">
       <c r="F276" s="7" t="n"/>
@@ -2864,6 +3164,7 @@
       <c r="J276" s="8" t="n"/>
       <c r="K276" s="8" t="n"/>
       <c r="L276" s="8" t="n"/>
+      <c r="M276" s="8" t="n"/>
     </row>
     <row r="277">
       <c r="F277" s="7" t="n"/>
@@ -2871,6 +3172,7 @@
       <c r="J277" s="8" t="n"/>
       <c r="K277" s="8" t="n"/>
       <c r="L277" s="8" t="n"/>
+      <c r="M277" s="8" t="n"/>
     </row>
     <row r="278">
       <c r="F278" s="7" t="n"/>
@@ -2878,6 +3180,7 @@
       <c r="J278" s="8" t="n"/>
       <c r="K278" s="8" t="n"/>
       <c r="L278" s="8" t="n"/>
+      <c r="M278" s="8" t="n"/>
     </row>
     <row r="279">
       <c r="F279" s="7" t="n"/>
@@ -2885,6 +3188,7 @@
       <c r="J279" s="8" t="n"/>
       <c r="K279" s="8" t="n"/>
       <c r="L279" s="8" t="n"/>
+      <c r="M279" s="8" t="n"/>
     </row>
     <row r="280">
       <c r="F280" s="7" t="n"/>
@@ -2892,6 +3196,7 @@
       <c r="J280" s="8" t="n"/>
       <c r="K280" s="8" t="n"/>
       <c r="L280" s="8" t="n"/>
+      <c r="M280" s="8" t="n"/>
     </row>
     <row r="281">
       <c r="F281" s="7" t="n"/>
@@ -2899,6 +3204,7 @@
       <c r="J281" s="8" t="n"/>
       <c r="K281" s="8" t="n"/>
       <c r="L281" s="8" t="n"/>
+      <c r="M281" s="8" t="n"/>
     </row>
     <row r="282">
       <c r="F282" s="7" t="n"/>
@@ -2906,6 +3212,7 @@
       <c r="J282" s="8" t="n"/>
       <c r="K282" s="8" t="n"/>
       <c r="L282" s="8" t="n"/>
+      <c r="M282" s="8" t="n"/>
     </row>
     <row r="283">
       <c r="F283" s="7" t="n"/>
@@ -2913,6 +3220,7 @@
       <c r="J283" s="8" t="n"/>
       <c r="K283" s="8" t="n"/>
       <c r="L283" s="8" t="n"/>
+      <c r="M283" s="8" t="n"/>
     </row>
     <row r="284">
       <c r="F284" s="7" t="n"/>
@@ -2920,6 +3228,7 @@
       <c r="J284" s="8" t="n"/>
       <c r="K284" s="8" t="n"/>
       <c r="L284" s="8" t="n"/>
+      <c r="M284" s="8" t="n"/>
     </row>
     <row r="285">
       <c r="F285" s="7" t="n"/>
@@ -2927,6 +3236,7 @@
       <c r="J285" s="8" t="n"/>
       <c r="K285" s="8" t="n"/>
       <c r="L285" s="8" t="n"/>
+      <c r="M285" s="8" t="n"/>
     </row>
     <row r="286">
       <c r="F286" s="7" t="n"/>
@@ -2934,6 +3244,7 @@
       <c r="J286" s="8" t="n"/>
       <c r="K286" s="8" t="n"/>
       <c r="L286" s="8" t="n"/>
+      <c r="M286" s="8" t="n"/>
     </row>
     <row r="287">
       <c r="F287" s="7" t="n"/>
@@ -2941,6 +3252,7 @@
       <c r="J287" s="8" t="n"/>
       <c r="K287" s="8" t="n"/>
       <c r="L287" s="8" t="n"/>
+      <c r="M287" s="8" t="n"/>
     </row>
     <row r="288">
       <c r="F288" s="7" t="n"/>
@@ -2948,6 +3260,7 @@
       <c r="J288" s="8" t="n"/>
       <c r="K288" s="8" t="n"/>
       <c r="L288" s="8" t="n"/>
+      <c r="M288" s="8" t="n"/>
     </row>
     <row r="289">
       <c r="F289" s="7" t="n"/>
@@ -2955,6 +3268,7 @@
       <c r="J289" s="8" t="n"/>
       <c r="K289" s="8" t="n"/>
       <c r="L289" s="8" t="n"/>
+      <c r="M289" s="8" t="n"/>
     </row>
     <row r="290">
       <c r="F290" s="7" t="n"/>
@@ -2962,6 +3276,7 @@
       <c r="J290" s="8" t="n"/>
       <c r="K290" s="8" t="n"/>
       <c r="L290" s="8" t="n"/>
+      <c r="M290" s="8" t="n"/>
     </row>
     <row r="291">
       <c r="F291" s="7" t="n"/>
@@ -2969,6 +3284,7 @@
       <c r="J291" s="8" t="n"/>
       <c r="K291" s="8" t="n"/>
       <c r="L291" s="8" t="n"/>
+      <c r="M291" s="8" t="n"/>
     </row>
     <row r="292">
       <c r="F292" s="7" t="n"/>
@@ -2976,6 +3292,7 @@
       <c r="J292" s="8" t="n"/>
       <c r="K292" s="8" t="n"/>
       <c r="L292" s="8" t="n"/>
+      <c r="M292" s="8" t="n"/>
     </row>
     <row r="293">
       <c r="F293" s="7" t="n"/>
@@ -2983,6 +3300,7 @@
       <c r="J293" s="8" t="n"/>
       <c r="K293" s="8" t="n"/>
       <c r="L293" s="8" t="n"/>
+      <c r="M293" s="8" t="n"/>
     </row>
     <row r="294">
       <c r="F294" s="7" t="n"/>
@@ -2990,6 +3308,7 @@
       <c r="J294" s="8" t="n"/>
       <c r="K294" s="8" t="n"/>
       <c r="L294" s="8" t="n"/>
+      <c r="M294" s="8" t="n"/>
     </row>
     <row r="295">
       <c r="F295" s="7" t="n"/>
@@ -2997,6 +3316,7 @@
       <c r="J295" s="8" t="n"/>
       <c r="K295" s="8" t="n"/>
       <c r="L295" s="8" t="n"/>
+      <c r="M295" s="8" t="n"/>
     </row>
     <row r="296">
       <c r="F296" s="7" t="n"/>
@@ -3004,6 +3324,7 @@
       <c r="J296" s="8" t="n"/>
       <c r="K296" s="8" t="n"/>
       <c r="L296" s="8" t="n"/>
+      <c r="M296" s="8" t="n"/>
     </row>
     <row r="297">
       <c r="F297" s="7" t="n"/>
@@ -3011,6 +3332,7 @@
       <c r="J297" s="8" t="n"/>
       <c r="K297" s="8" t="n"/>
       <c r="L297" s="8" t="n"/>
+      <c r="M297" s="8" t="n"/>
     </row>
     <row r="298">
       <c r="F298" s="7" t="n"/>
@@ -3018,6 +3340,7 @@
       <c r="J298" s="8" t="n"/>
       <c r="K298" s="8" t="n"/>
       <c r="L298" s="8" t="n"/>
+      <c r="M298" s="8" t="n"/>
     </row>
     <row r="299">
       <c r="F299" s="7" t="n"/>
@@ -3025,6 +3348,7 @@
       <c r="J299" s="8" t="n"/>
       <c r="K299" s="8" t="n"/>
       <c r="L299" s="8" t="n"/>
+      <c r="M299" s="8" t="n"/>
     </row>
     <row r="300">
       <c r="F300" s="7" t="n"/>
@@ -3032,6 +3356,7 @@
       <c r="J300" s="8" t="n"/>
       <c r="K300" s="8" t="n"/>
       <c r="L300" s="8" t="n"/>
+      <c r="M300" s="8" t="n"/>
     </row>
     <row r="301">
       <c r="F301" s="7" t="n"/>
@@ -3039,6 +3364,7 @@
       <c r="J301" s="8" t="n"/>
       <c r="K301" s="8" t="n"/>
       <c r="L301" s="8" t="n"/>
+      <c r="M301" s="8" t="n"/>
     </row>
     <row r="302">
       <c r="F302" s="7" t="n"/>
@@ -3046,6 +3372,7 @@
       <c r="J302" s="8" t="n"/>
       <c r="K302" s="8" t="n"/>
       <c r="L302" s="8" t="n"/>
+      <c r="M302" s="8" t="n"/>
     </row>
     <row r="303">
       <c r="F303" s="7" t="n"/>
@@ -3053,6 +3380,7 @@
       <c r="J303" s="8" t="n"/>
       <c r="K303" s="8" t="n"/>
       <c r="L303" s="8" t="n"/>
+      <c r="M303" s="8" t="n"/>
     </row>
     <row r="304">
       <c r="F304" s="7" t="n"/>
@@ -3060,6 +3388,7 @@
       <c r="J304" s="8" t="n"/>
       <c r="K304" s="8" t="n"/>
       <c r="L304" s="8" t="n"/>
+      <c r="M304" s="8" t="n"/>
     </row>
     <row r="305">
       <c r="F305" s="7" t="n"/>
@@ -3067,6 +3396,7 @@
       <c r="J305" s="8" t="n"/>
       <c r="K305" s="8" t="n"/>
       <c r="L305" s="8" t="n"/>
+      <c r="M305" s="8" t="n"/>
     </row>
     <row r="306">
       <c r="F306" s="7" t="n"/>
@@ -3074,6 +3404,7 @@
       <c r="J306" s="8" t="n"/>
       <c r="K306" s="8" t="n"/>
       <c r="L306" s="8" t="n"/>
+      <c r="M306" s="8" t="n"/>
     </row>
     <row r="307">
       <c r="F307" s="7" t="n"/>
@@ -3081,6 +3412,7 @@
       <c r="J307" s="8" t="n"/>
       <c r="K307" s="8" t="n"/>
       <c r="L307" s="8" t="n"/>
+      <c r="M307" s="8" t="n"/>
     </row>
     <row r="308">
       <c r="F308" s="7" t="n"/>
@@ -3088,6 +3420,7 @@
       <c r="J308" s="8" t="n"/>
       <c r="K308" s="8" t="n"/>
       <c r="L308" s="8" t="n"/>
+      <c r="M308" s="8" t="n"/>
     </row>
     <row r="309">
       <c r="F309" s="7" t="n"/>
@@ -3095,6 +3428,7 @@
       <c r="J309" s="8" t="n"/>
       <c r="K309" s="8" t="n"/>
       <c r="L309" s="8" t="n"/>
+      <c r="M309" s="8" t="n"/>
     </row>
     <row r="310">
       <c r="F310" s="7" t="n"/>
@@ -3102,6 +3436,7 @@
       <c r="J310" s="8" t="n"/>
       <c r="K310" s="8" t="n"/>
       <c r="L310" s="8" t="n"/>
+      <c r="M310" s="8" t="n"/>
     </row>
     <row r="311">
       <c r="F311" s="7" t="n"/>
@@ -3109,6 +3444,7 @@
       <c r="J311" s="8" t="n"/>
       <c r="K311" s="8" t="n"/>
       <c r="L311" s="8" t="n"/>
+      <c r="M311" s="8" t="n"/>
     </row>
     <row r="312">
       <c r="F312" s="7" t="n"/>
@@ -3116,6 +3452,7 @@
       <c r="J312" s="8" t="n"/>
       <c r="K312" s="8" t="n"/>
       <c r="L312" s="8" t="n"/>
+      <c r="M312" s="8" t="n"/>
     </row>
     <row r="313">
       <c r="F313" s="7" t="n"/>
@@ -3123,6 +3460,7 @@
       <c r="J313" s="8" t="n"/>
       <c r="K313" s="8" t="n"/>
       <c r="L313" s="8" t="n"/>
+      <c r="M313" s="8" t="n"/>
     </row>
     <row r="314">
       <c r="F314" s="7" t="n"/>
@@ -3130,6 +3468,7 @@
       <c r="J314" s="8" t="n"/>
       <c r="K314" s="8" t="n"/>
       <c r="L314" s="8" t="n"/>
+      <c r="M314" s="8" t="n"/>
     </row>
     <row r="315">
       <c r="F315" s="7" t="n"/>
@@ -3137,6 +3476,7 @@
       <c r="J315" s="8" t="n"/>
       <c r="K315" s="8" t="n"/>
       <c r="L315" s="8" t="n"/>
+      <c r="M315" s="8" t="n"/>
     </row>
     <row r="316">
       <c r="F316" s="7" t="n"/>
@@ -3144,6 +3484,7 @@
       <c r="J316" s="8" t="n"/>
       <c r="K316" s="8" t="n"/>
       <c r="L316" s="8" t="n"/>
+      <c r="M316" s="8" t="n"/>
     </row>
     <row r="317">
       <c r="F317" s="7" t="n"/>
@@ -3151,6 +3492,7 @@
       <c r="J317" s="8" t="n"/>
       <c r="K317" s="8" t="n"/>
       <c r="L317" s="8" t="n"/>
+      <c r="M317" s="8" t="n"/>
     </row>
     <row r="318">
       <c r="F318" s="7" t="n"/>
@@ -3158,6 +3500,7 @@
       <c r="J318" s="8" t="n"/>
       <c r="K318" s="8" t="n"/>
       <c r="L318" s="8" t="n"/>
+      <c r="M318" s="8" t="n"/>
     </row>
     <row r="319">
       <c r="F319" s="7" t="n"/>
@@ -3165,6 +3508,7 @@
       <c r="J319" s="8" t="n"/>
       <c r="K319" s="8" t="n"/>
       <c r="L319" s="8" t="n"/>
+      <c r="M319" s="8" t="n"/>
     </row>
     <row r="320">
       <c r="F320" s="7" t="n"/>
@@ -3172,6 +3516,7 @@
       <c r="J320" s="8" t="n"/>
       <c r="K320" s="8" t="n"/>
       <c r="L320" s="8" t="n"/>
+      <c r="M320" s="8" t="n"/>
     </row>
     <row r="321">
       <c r="F321" s="7" t="n"/>
@@ -3179,6 +3524,7 @@
       <c r="J321" s="8" t="n"/>
       <c r="K321" s="8" t="n"/>
       <c r="L321" s="8" t="n"/>
+      <c r="M321" s="8" t="n"/>
     </row>
     <row r="322">
       <c r="F322" s="7" t="n"/>
@@ -3186,6 +3532,7 @@
       <c r="J322" s="8" t="n"/>
       <c r="K322" s="8" t="n"/>
       <c r="L322" s="8" t="n"/>
+      <c r="M322" s="8" t="n"/>
     </row>
     <row r="323">
       <c r="F323" s="7" t="n"/>
@@ -3193,6 +3540,7 @@
       <c r="J323" s="8" t="n"/>
       <c r="K323" s="8" t="n"/>
       <c r="L323" s="8" t="n"/>
+      <c r="M323" s="8" t="n"/>
     </row>
     <row r="324">
       <c r="F324" s="7" t="n"/>
@@ -3200,6 +3548,7 @@
       <c r="J324" s="8" t="n"/>
       <c r="K324" s="8" t="n"/>
       <c r="L324" s="8" t="n"/>
+      <c r="M324" s="8" t="n"/>
     </row>
     <row r="325">
       <c r="F325" s="7" t="n"/>
@@ -3207,6 +3556,7 @@
       <c r="J325" s="8" t="n"/>
       <c r="K325" s="8" t="n"/>
       <c r="L325" s="8" t="n"/>
+      <c r="M325" s="8" t="n"/>
     </row>
     <row r="326">
       <c r="F326" s="7" t="n"/>
@@ -3214,6 +3564,7 @@
       <c r="J326" s="8" t="n"/>
       <c r="K326" s="8" t="n"/>
       <c r="L326" s="8" t="n"/>
+      <c r="M326" s="8" t="n"/>
     </row>
     <row r="327">
       <c r="F327" s="7" t="n"/>
@@ -3221,6 +3572,7 @@
       <c r="J327" s="8" t="n"/>
       <c r="K327" s="8" t="n"/>
       <c r="L327" s="8" t="n"/>
+      <c r="M327" s="8" t="n"/>
     </row>
     <row r="328">
       <c r="F328" s="7" t="n"/>
@@ -3228,6 +3580,7 @@
       <c r="J328" s="8" t="n"/>
       <c r="K328" s="8" t="n"/>
       <c r="L328" s="8" t="n"/>
+      <c r="M328" s="8" t="n"/>
     </row>
     <row r="329">
       <c r="F329" s="7" t="n"/>
@@ -3235,6 +3588,7 @@
       <c r="J329" s="8" t="n"/>
       <c r="K329" s="8" t="n"/>
       <c r="L329" s="8" t="n"/>
+      <c r="M329" s="8" t="n"/>
     </row>
     <row r="330">
       <c r="F330" s="7" t="n"/>
@@ -3242,6 +3596,7 @@
       <c r="J330" s="8" t="n"/>
       <c r="K330" s="8" t="n"/>
       <c r="L330" s="8" t="n"/>
+      <c r="M330" s="8" t="n"/>
     </row>
     <row r="331">
       <c r="F331" s="7" t="n"/>
@@ -3249,6 +3604,7 @@
       <c r="J331" s="8" t="n"/>
       <c r="K331" s="8" t="n"/>
       <c r="L331" s="8" t="n"/>
+      <c r="M331" s="8" t="n"/>
     </row>
     <row r="332">
       <c r="F332" s="7" t="n"/>
@@ -3256,6 +3612,7 @@
       <c r="J332" s="8" t="n"/>
       <c r="K332" s="8" t="n"/>
       <c r="L332" s="8" t="n"/>
+      <c r="M332" s="8" t="n"/>
     </row>
     <row r="333">
       <c r="F333" s="7" t="n"/>
@@ -3263,6 +3620,7 @@
       <c r="J333" s="8" t="n"/>
       <c r="K333" s="8" t="n"/>
       <c r="L333" s="8" t="n"/>
+      <c r="M333" s="8" t="n"/>
     </row>
     <row r="334">
       <c r="F334" s="7" t="n"/>
@@ -3270,6 +3628,7 @@
       <c r="J334" s="8" t="n"/>
       <c r="K334" s="8" t="n"/>
       <c r="L334" s="8" t="n"/>
+      <c r="M334" s="8" t="n"/>
     </row>
     <row r="335">
       <c r="F335" s="7" t="n"/>
@@ -3277,6 +3636,7 @@
       <c r="J335" s="8" t="n"/>
       <c r="K335" s="8" t="n"/>
       <c r="L335" s="8" t="n"/>
+      <c r="M335" s="8" t="n"/>
     </row>
     <row r="336">
       <c r="F336" s="7" t="n"/>
@@ -3284,6 +3644,7 @@
       <c r="J336" s="8" t="n"/>
       <c r="K336" s="8" t="n"/>
       <c r="L336" s="8" t="n"/>
+      <c r="M336" s="8" t="n"/>
     </row>
     <row r="337">
       <c r="F337" s="7" t="n"/>
@@ -3291,6 +3652,7 @@
       <c r="J337" s="8" t="n"/>
       <c r="K337" s="8" t="n"/>
       <c r="L337" s="8" t="n"/>
+      <c r="M337" s="8" t="n"/>
     </row>
     <row r="338">
       <c r="F338" s="7" t="n"/>
@@ -3298,6 +3660,7 @@
       <c r="J338" s="8" t="n"/>
       <c r="K338" s="8" t="n"/>
       <c r="L338" s="8" t="n"/>
+      <c r="M338" s="8" t="n"/>
     </row>
     <row r="339">
       <c r="F339" s="7" t="n"/>
@@ -3305,6 +3668,7 @@
       <c r="J339" s="8" t="n"/>
       <c r="K339" s="8" t="n"/>
       <c r="L339" s="8" t="n"/>
+      <c r="M339" s="8" t="n"/>
     </row>
     <row r="340">
       <c r="F340" s="7" t="n"/>
@@ -3312,6 +3676,7 @@
       <c r="J340" s="8" t="n"/>
       <c r="K340" s="8" t="n"/>
       <c r="L340" s="8" t="n"/>
+      <c r="M340" s="8" t="n"/>
     </row>
     <row r="341">
       <c r="F341" s="7" t="n"/>
@@ -3319,6 +3684,7 @@
       <c r="J341" s="8" t="n"/>
       <c r="K341" s="8" t="n"/>
       <c r="L341" s="8" t="n"/>
+      <c r="M341" s="8" t="n"/>
     </row>
     <row r="342">
       <c r="F342" s="7" t="n"/>
@@ -3326,6 +3692,7 @@
       <c r="J342" s="8" t="n"/>
       <c r="K342" s="8" t="n"/>
       <c r="L342" s="8" t="n"/>
+      <c r="M342" s="8" t="n"/>
     </row>
     <row r="343">
       <c r="F343" s="7" t="n"/>
@@ -3333,6 +3700,7 @@
       <c r="J343" s="8" t="n"/>
       <c r="K343" s="8" t="n"/>
       <c r="L343" s="8" t="n"/>
+      <c r="M343" s="8" t="n"/>
     </row>
     <row r="344">
       <c r="F344" s="7" t="n"/>
@@ -3340,6 +3708,7 @@
       <c r="J344" s="8" t="n"/>
       <c r="K344" s="8" t="n"/>
       <c r="L344" s="8" t="n"/>
+      <c r="M344" s="8" t="n"/>
     </row>
     <row r="345">
       <c r="F345" s="7" t="n"/>
@@ -3347,6 +3716,7 @@
       <c r="J345" s="8" t="n"/>
       <c r="K345" s="8" t="n"/>
       <c r="L345" s="8" t="n"/>
+      <c r="M345" s="8" t="n"/>
     </row>
     <row r="346">
       <c r="F346" s="7" t="n"/>
@@ -3354,6 +3724,7 @@
       <c r="J346" s="8" t="n"/>
       <c r="K346" s="8" t="n"/>
       <c r="L346" s="8" t="n"/>
+      <c r="M346" s="8" t="n"/>
     </row>
     <row r="347">
       <c r="F347" s="7" t="n"/>
@@ -3361,6 +3732,7 @@
       <c r="J347" s="8" t="n"/>
       <c r="K347" s="8" t="n"/>
       <c r="L347" s="8" t="n"/>
+      <c r="M347" s="8" t="n"/>
     </row>
     <row r="348">
       <c r="F348" s="7" t="n"/>
@@ -3368,6 +3740,7 @@
       <c r="J348" s="8" t="n"/>
       <c r="K348" s="8" t="n"/>
       <c r="L348" s="8" t="n"/>
+      <c r="M348" s="8" t="n"/>
     </row>
     <row r="349">
       <c r="F349" s="7" t="n"/>
@@ -3375,6 +3748,7 @@
       <c r="J349" s="8" t="n"/>
       <c r="K349" s="8" t="n"/>
       <c r="L349" s="8" t="n"/>
+      <c r="M349" s="8" t="n"/>
     </row>
     <row r="350">
       <c r="F350" s="7" t="n"/>
@@ -3382,6 +3756,7 @@
       <c r="J350" s="8" t="n"/>
       <c r="K350" s="8" t="n"/>
       <c r="L350" s="8" t="n"/>
+      <c r="M350" s="8" t="n"/>
     </row>
     <row r="351">
       <c r="F351" s="7" t="n"/>
@@ -3389,6 +3764,7 @@
       <c r="J351" s="8" t="n"/>
       <c r="K351" s="8" t="n"/>
       <c r="L351" s="8" t="n"/>
+      <c r="M351" s="8" t="n"/>
     </row>
     <row r="352">
       <c r="F352" s="7" t="n"/>
@@ -3396,6 +3772,7 @@
       <c r="J352" s="8" t="n"/>
       <c r="K352" s="8" t="n"/>
       <c r="L352" s="8" t="n"/>
+      <c r="M352" s="8" t="n"/>
     </row>
     <row r="353">
       <c r="F353" s="7" t="n"/>
@@ -3403,6 +3780,7 @@
       <c r="J353" s="8" t="n"/>
       <c r="K353" s="8" t="n"/>
       <c r="L353" s="8" t="n"/>
+      <c r="M353" s="8" t="n"/>
     </row>
     <row r="354">
       <c r="F354" s="7" t="n"/>
@@ -3410,6 +3788,7 @@
       <c r="J354" s="8" t="n"/>
       <c r="K354" s="8" t="n"/>
       <c r="L354" s="8" t="n"/>
+      <c r="M354" s="8" t="n"/>
     </row>
     <row r="355">
       <c r="F355" s="7" t="n"/>
@@ -3417,6 +3796,7 @@
       <c r="J355" s="8" t="n"/>
       <c r="K355" s="8" t="n"/>
       <c r="L355" s="8" t="n"/>
+      <c r="M355" s="8" t="n"/>
     </row>
     <row r="356">
       <c r="F356" s="7" t="n"/>
@@ -3424,6 +3804,7 @@
       <c r="J356" s="8" t="n"/>
       <c r="K356" s="8" t="n"/>
       <c r="L356" s="8" t="n"/>
+      <c r="M356" s="8" t="n"/>
     </row>
     <row r="357">
       <c r="F357" s="7" t="n"/>
@@ -3431,6 +3812,7 @@
       <c r="J357" s="8" t="n"/>
       <c r="K357" s="8" t="n"/>
       <c r="L357" s="8" t="n"/>
+      <c r="M357" s="8" t="n"/>
     </row>
     <row r="358">
       <c r="F358" s="7" t="n"/>
@@ -3438,6 +3820,7 @@
       <c r="J358" s="8" t="n"/>
       <c r="K358" s="8" t="n"/>
       <c r="L358" s="8" t="n"/>
+      <c r="M358" s="8" t="n"/>
     </row>
     <row r="359">
       <c r="F359" s="7" t="n"/>
@@ -3445,6 +3828,7 @@
       <c r="J359" s="8" t="n"/>
       <c r="K359" s="8" t="n"/>
       <c r="L359" s="8" t="n"/>
+      <c r="M359" s="8" t="n"/>
     </row>
     <row r="360">
       <c r="F360" s="7" t="n"/>
@@ -3452,6 +3836,7 @@
       <c r="J360" s="8" t="n"/>
       <c r="K360" s="8" t="n"/>
       <c r="L360" s="8" t="n"/>
+      <c r="M360" s="8" t="n"/>
     </row>
     <row r="361">
       <c r="F361" s="7" t="n"/>
@@ -3459,6 +3844,7 @@
       <c r="J361" s="8" t="n"/>
       <c r="K361" s="8" t="n"/>
       <c r="L361" s="8" t="n"/>
+      <c r="M361" s="8" t="n"/>
     </row>
     <row r="362">
       <c r="F362" s="7" t="n"/>
@@ -3466,6 +3852,7 @@
       <c r="J362" s="8" t="n"/>
       <c r="K362" s="8" t="n"/>
       <c r="L362" s="8" t="n"/>
+      <c r="M362" s="8" t="n"/>
     </row>
     <row r="363">
       <c r="F363" s="7" t="n"/>
@@ -3473,6 +3860,7 @@
       <c r="J363" s="8" t="n"/>
       <c r="K363" s="8" t="n"/>
       <c r="L363" s="8" t="n"/>
+      <c r="M363" s="8" t="n"/>
     </row>
     <row r="364">
       <c r="F364" s="7" t="n"/>
@@ -3480,6 +3868,7 @@
       <c r="J364" s="8" t="n"/>
       <c r="K364" s="8" t="n"/>
       <c r="L364" s="8" t="n"/>
+      <c r="M364" s="8" t="n"/>
     </row>
     <row r="365">
       <c r="F365" s="7" t="n"/>
@@ -3487,6 +3876,7 @@
       <c r="J365" s="8" t="n"/>
       <c r="K365" s="8" t="n"/>
       <c r="L365" s="8" t="n"/>
+      <c r="M365" s="8" t="n"/>
     </row>
     <row r="366">
       <c r="F366" s="7" t="n"/>
@@ -3494,6 +3884,7 @@
       <c r="J366" s="8" t="n"/>
       <c r="K366" s="8" t="n"/>
       <c r="L366" s="8" t="n"/>
+      <c r="M366" s="8" t="n"/>
     </row>
     <row r="367">
       <c r="F367" s="7" t="n"/>
@@ -3501,6 +3892,7 @@
       <c r="J367" s="8" t="n"/>
       <c r="K367" s="8" t="n"/>
       <c r="L367" s="8" t="n"/>
+      <c r="M367" s="8" t="n"/>
     </row>
     <row r="368">
       <c r="F368" s="7" t="n"/>
@@ -3508,6 +3900,7 @@
       <c r="J368" s="8" t="n"/>
       <c r="K368" s="8" t="n"/>
       <c r="L368" s="8" t="n"/>
+      <c r="M368" s="8" t="n"/>
     </row>
     <row r="369">
       <c r="F369" s="7" t="n"/>
@@ -3515,6 +3908,7 @@
       <c r="J369" s="8" t="n"/>
       <c r="K369" s="8" t="n"/>
       <c r="L369" s="8" t="n"/>
+      <c r="M369" s="8" t="n"/>
     </row>
     <row r="370">
       <c r="F370" s="7" t="n"/>
@@ -3522,6 +3916,7 @@
       <c r="J370" s="8" t="n"/>
       <c r="K370" s="8" t="n"/>
       <c r="L370" s="8" t="n"/>
+      <c r="M370" s="8" t="n"/>
     </row>
     <row r="371">
       <c r="F371" s="7" t="n"/>
@@ -3529,6 +3924,7 @@
       <c r="J371" s="8" t="n"/>
       <c r="K371" s="8" t="n"/>
       <c r="L371" s="8" t="n"/>
+      <c r="M371" s="8" t="n"/>
     </row>
     <row r="372">
       <c r="F372" s="7" t="n"/>
@@ -3536,6 +3932,7 @@
       <c r="J372" s="8" t="n"/>
       <c r="K372" s="8" t="n"/>
       <c r="L372" s="8" t="n"/>
+      <c r="M372" s="8" t="n"/>
     </row>
     <row r="373">
       <c r="F373" s="7" t="n"/>
@@ -3543,6 +3940,7 @@
       <c r="J373" s="8" t="n"/>
       <c r="K373" s="8" t="n"/>
       <c r="L373" s="8" t="n"/>
+      <c r="M373" s="8" t="n"/>
     </row>
     <row r="374">
       <c r="F374" s="7" t="n"/>
@@ -3550,6 +3948,7 @@
       <c r="J374" s="8" t="n"/>
       <c r="K374" s="8" t="n"/>
       <c r="L374" s="8" t="n"/>
+      <c r="M374" s="8" t="n"/>
     </row>
     <row r="375">
       <c r="F375" s="7" t="n"/>
@@ -3557,6 +3956,7 @@
       <c r="J375" s="8" t="n"/>
       <c r="K375" s="8" t="n"/>
       <c r="L375" s="8" t="n"/>
+      <c r="M375" s="8" t="n"/>
     </row>
     <row r="376">
       <c r="F376" s="7" t="n"/>
@@ -3564,6 +3964,7 @@
       <c r="J376" s="8" t="n"/>
       <c r="K376" s="8" t="n"/>
       <c r="L376" s="8" t="n"/>
+      <c r="M376" s="8" t="n"/>
     </row>
     <row r="377">
       <c r="F377" s="7" t="n"/>
@@ -3571,6 +3972,7 @@
       <c r="J377" s="8" t="n"/>
       <c r="K377" s="8" t="n"/>
       <c r="L377" s="8" t="n"/>
+      <c r="M377" s="8" t="n"/>
     </row>
     <row r="378">
       <c r="F378" s="7" t="n"/>
@@ -3578,6 +3980,7 @@
       <c r="J378" s="8" t="n"/>
       <c r="K378" s="8" t="n"/>
       <c r="L378" s="8" t="n"/>
+      <c r="M378" s="8" t="n"/>
     </row>
     <row r="379">
       <c r="F379" s="7" t="n"/>
@@ -3585,6 +3988,7 @@
       <c r="J379" s="8" t="n"/>
       <c r="K379" s="8" t="n"/>
       <c r="L379" s="8" t="n"/>
+      <c r="M379" s="8" t="n"/>
     </row>
     <row r="380">
       <c r="F380" s="7" t="n"/>
@@ -3592,6 +3996,7 @@
       <c r="J380" s="8" t="n"/>
       <c r="K380" s="8" t="n"/>
       <c r="L380" s="8" t="n"/>
+      <c r="M380" s="8" t="n"/>
     </row>
     <row r="381">
       <c r="F381" s="7" t="n"/>
@@ -3599,6 +4004,7 @@
       <c r="J381" s="8" t="n"/>
       <c r="K381" s="8" t="n"/>
       <c r="L381" s="8" t="n"/>
+      <c r="M381" s="8" t="n"/>
     </row>
     <row r="382">
       <c r="F382" s="7" t="n"/>
@@ -3606,6 +4012,7 @@
       <c r="J382" s="8" t="n"/>
       <c r="K382" s="8" t="n"/>
       <c r="L382" s="8" t="n"/>
+      <c r="M382" s="8" t="n"/>
     </row>
     <row r="383">
       <c r="F383" s="7" t="n"/>
@@ -3613,6 +4020,7 @@
       <c r="J383" s="8" t="n"/>
       <c r="K383" s="8" t="n"/>
       <c r="L383" s="8" t="n"/>
+      <c r="M383" s="8" t="n"/>
     </row>
     <row r="384">
       <c r="F384" s="7" t="n"/>
@@ -3620,6 +4028,7 @@
       <c r="J384" s="8" t="n"/>
       <c r="K384" s="8" t="n"/>
       <c r="L384" s="8" t="n"/>
+      <c r="M384" s="8" t="n"/>
     </row>
     <row r="385">
       <c r="F385" s="7" t="n"/>
@@ -3627,6 +4036,7 @@
       <c r="J385" s="8" t="n"/>
       <c r="K385" s="8" t="n"/>
       <c r="L385" s="8" t="n"/>
+      <c r="M385" s="8" t="n"/>
     </row>
     <row r="386">
       <c r="F386" s="7" t="n"/>
@@ -3634,6 +4044,7 @@
       <c r="J386" s="8" t="n"/>
       <c r="K386" s="8" t="n"/>
       <c r="L386" s="8" t="n"/>
+      <c r="M386" s="8" t="n"/>
     </row>
     <row r="387">
       <c r="F387" s="7" t="n"/>
@@ -3641,6 +4052,7 @@
       <c r="J387" s="8" t="n"/>
       <c r="K387" s="8" t="n"/>
       <c r="L387" s="8" t="n"/>
+      <c r="M387" s="8" t="n"/>
     </row>
     <row r="388">
       <c r="F388" s="7" t="n"/>
@@ -3648,6 +4060,7 @@
       <c r="J388" s="8" t="n"/>
       <c r="K388" s="8" t="n"/>
       <c r="L388" s="8" t="n"/>
+      <c r="M388" s="8" t="n"/>
     </row>
     <row r="389">
       <c r="F389" s="7" t="n"/>
@@ -3655,6 +4068,7 @@
       <c r="J389" s="8" t="n"/>
       <c r="K389" s="8" t="n"/>
       <c r="L389" s="8" t="n"/>
+      <c r="M389" s="8" t="n"/>
     </row>
     <row r="390">
       <c r="F390" s="7" t="n"/>
@@ -3662,6 +4076,7 @@
       <c r="J390" s="8" t="n"/>
       <c r="K390" s="8" t="n"/>
       <c r="L390" s="8" t="n"/>
+      <c r="M390" s="8" t="n"/>
     </row>
     <row r="391">
       <c r="F391" s="7" t="n"/>
@@ -3669,6 +4084,7 @@
       <c r="J391" s="8" t="n"/>
       <c r="K391" s="8" t="n"/>
       <c r="L391" s="8" t="n"/>
+      <c r="M391" s="8" t="n"/>
     </row>
     <row r="392">
       <c r="F392" s="7" t="n"/>
@@ -3676,6 +4092,7 @@
       <c r="J392" s="8" t="n"/>
       <c r="K392" s="8" t="n"/>
       <c r="L392" s="8" t="n"/>
+      <c r="M392" s="8" t="n"/>
     </row>
     <row r="393">
       <c r="F393" s="7" t="n"/>
@@ -3683,6 +4100,7 @@
       <c r="J393" s="8" t="n"/>
       <c r="K393" s="8" t="n"/>
       <c r="L393" s="8" t="n"/>
+      <c r="M393" s="8" t="n"/>
     </row>
     <row r="394">
       <c r="F394" s="7" t="n"/>
@@ -3690,6 +4108,7 @@
       <c r="J394" s="8" t="n"/>
       <c r="K394" s="8" t="n"/>
       <c r="L394" s="8" t="n"/>
+      <c r="M394" s="8" t="n"/>
     </row>
     <row r="395">
       <c r="F395" s="7" t="n"/>
@@ -3697,6 +4116,7 @@
       <c r="J395" s="8" t="n"/>
       <c r="K395" s="8" t="n"/>
       <c r="L395" s="8" t="n"/>
+      <c r="M395" s="8" t="n"/>
     </row>
     <row r="396">
       <c r="F396" s="7" t="n"/>
@@ -3704,6 +4124,7 @@
       <c r="J396" s="8" t="n"/>
       <c r="K396" s="8" t="n"/>
       <c r="L396" s="8" t="n"/>
+      <c r="M396" s="8" t="n"/>
     </row>
     <row r="397">
       <c r="F397" s="7" t="n"/>
@@ -3711,6 +4132,7 @@
       <c r="J397" s="8" t="n"/>
       <c r="K397" s="8" t="n"/>
       <c r="L397" s="8" t="n"/>
+      <c r="M397" s="8" t="n"/>
     </row>
     <row r="398">
       <c r="F398" s="7" t="n"/>
@@ -3718,6 +4140,7 @@
       <c r="J398" s="8" t="n"/>
       <c r="K398" s="8" t="n"/>
       <c r="L398" s="8" t="n"/>
+      <c r="M398" s="8" t="n"/>
     </row>
     <row r="399">
       <c r="F399" s="7" t="n"/>
@@ -3725,6 +4148,7 @@
       <c r="J399" s="8" t="n"/>
       <c r="K399" s="8" t="n"/>
       <c r="L399" s="8" t="n"/>
+      <c r="M399" s="8" t="n"/>
     </row>
     <row r="400">
       <c r="F400" s="7" t="n"/>
@@ -3732,6 +4156,7 @@
       <c r="J400" s="8" t="n"/>
       <c r="K400" s="8" t="n"/>
       <c r="L400" s="8" t="n"/>
+      <c r="M400" s="8" t="n"/>
     </row>
     <row r="401">
       <c r="F401" s="7" t="n"/>
@@ -3739,6 +4164,7 @@
       <c r="J401" s="8" t="n"/>
       <c r="K401" s="8" t="n"/>
       <c r="L401" s="8" t="n"/>
+      <c r="M401" s="8" t="n"/>
     </row>
     <row r="402">
       <c r="F402" s="7" t="n"/>
@@ -3746,6 +4172,7 @@
       <c r="J402" s="8" t="n"/>
       <c r="K402" s="8" t="n"/>
       <c r="L402" s="8" t="n"/>
+      <c r="M402" s="8" t="n"/>
     </row>
     <row r="403">
       <c r="F403" s="7" t="n"/>
@@ -3753,6 +4180,7 @@
       <c r="J403" s="8" t="n"/>
       <c r="K403" s="8" t="n"/>
       <c r="L403" s="8" t="n"/>
+      <c r="M403" s="8" t="n"/>
     </row>
     <row r="404">
       <c r="F404" s="7" t="n"/>
@@ -3760,6 +4188,7 @@
       <c r="J404" s="8" t="n"/>
       <c r="K404" s="8" t="n"/>
       <c r="L404" s="8" t="n"/>
+      <c r="M404" s="8" t="n"/>
     </row>
     <row r="405">
       <c r="F405" s="7" t="n"/>
@@ -3767,6 +4196,7 @@
       <c r="J405" s="8" t="n"/>
       <c r="K405" s="8" t="n"/>
       <c r="L405" s="8" t="n"/>
+      <c r="M405" s="8" t="n"/>
     </row>
     <row r="406">
       <c r="F406" s="7" t="n"/>
@@ -3774,6 +4204,7 @@
       <c r="J406" s="8" t="n"/>
       <c r="K406" s="8" t="n"/>
       <c r="L406" s="8" t="n"/>
+      <c r="M406" s="8" t="n"/>
     </row>
     <row r="407">
       <c r="F407" s="7" t="n"/>
@@ -3781,6 +4212,7 @@
       <c r="J407" s="8" t="n"/>
       <c r="K407" s="8" t="n"/>
       <c r="L407" s="8" t="n"/>
+      <c r="M407" s="8" t="n"/>
     </row>
     <row r="408">
       <c r="F408" s="7" t="n"/>
@@ -3788,6 +4220,7 @@
       <c r="J408" s="8" t="n"/>
       <c r="K408" s="8" t="n"/>
       <c r="L408" s="8" t="n"/>
+      <c r="M408" s="8" t="n"/>
     </row>
     <row r="409">
       <c r="F409" s="7" t="n"/>
@@ -3795,6 +4228,7 @@
       <c r="J409" s="8" t="n"/>
       <c r="K409" s="8" t="n"/>
       <c r="L409" s="8" t="n"/>
+      <c r="M409" s="8" t="n"/>
     </row>
     <row r="410">
       <c r="F410" s="7" t="n"/>
@@ -3802,6 +4236,7 @@
       <c r="J410" s="8" t="n"/>
       <c r="K410" s="8" t="n"/>
       <c r="L410" s="8" t="n"/>
+      <c r="M410" s="8" t="n"/>
     </row>
     <row r="411">
       <c r="F411" s="7" t="n"/>
@@ -3809,6 +4244,7 @@
       <c r="J411" s="8" t="n"/>
       <c r="K411" s="8" t="n"/>
       <c r="L411" s="8" t="n"/>
+      <c r="M411" s="8" t="n"/>
     </row>
     <row r="412">
       <c r="F412" s="7" t="n"/>
@@ -3816,6 +4252,7 @@
       <c r="J412" s="8" t="n"/>
       <c r="K412" s="8" t="n"/>
       <c r="L412" s="8" t="n"/>
+      <c r="M412" s="8" t="n"/>
     </row>
     <row r="413">
       <c r="F413" s="7" t="n"/>
@@ -3823,6 +4260,7 @@
       <c r="J413" s="8" t="n"/>
       <c r="K413" s="8" t="n"/>
       <c r="L413" s="8" t="n"/>
+      <c r="M413" s="8" t="n"/>
     </row>
     <row r="414">
       <c r="F414" s="7" t="n"/>
@@ -3830,6 +4268,7 @@
       <c r="J414" s="8" t="n"/>
       <c r="K414" s="8" t="n"/>
       <c r="L414" s="8" t="n"/>
+      <c r="M414" s="8" t="n"/>
     </row>
     <row r="415">
       <c r="F415" s="7" t="n"/>
@@ -3837,6 +4276,7 @@
       <c r="J415" s="8" t="n"/>
       <c r="K415" s="8" t="n"/>
       <c r="L415" s="8" t="n"/>
+      <c r="M415" s="8" t="n"/>
     </row>
     <row r="416">
       <c r="F416" s="7" t="n"/>
@@ -3844,6 +4284,7 @@
       <c r="J416" s="8" t="n"/>
       <c r="K416" s="8" t="n"/>
       <c r="L416" s="8" t="n"/>
+      <c r="M416" s="8" t="n"/>
     </row>
     <row r="417">
       <c r="F417" s="7" t="n"/>
@@ -3851,6 +4292,7 @@
       <c r="J417" s="8" t="n"/>
       <c r="K417" s="8" t="n"/>
       <c r="L417" s="8" t="n"/>
+      <c r="M417" s="8" t="n"/>
     </row>
     <row r="418">
       <c r="F418" s="7" t="n"/>
@@ -3858,6 +4300,7 @@
       <c r="J418" s="8" t="n"/>
       <c r="K418" s="8" t="n"/>
       <c r="L418" s="8" t="n"/>
+      <c r="M418" s="8" t="n"/>
     </row>
     <row r="419">
       <c r="F419" s="7" t="n"/>
@@ -3865,6 +4308,7 @@
       <c r="J419" s="8" t="n"/>
       <c r="K419" s="8" t="n"/>
       <c r="L419" s="8" t="n"/>
+      <c r="M419" s="8" t="n"/>
     </row>
     <row r="420">
       <c r="F420" s="7" t="n"/>
@@ -3872,6 +4316,7 @@
       <c r="J420" s="8" t="n"/>
       <c r="K420" s="8" t="n"/>
       <c r="L420" s="8" t="n"/>
+      <c r="M420" s="8" t="n"/>
     </row>
     <row r="421">
       <c r="F421" s="7" t="n"/>
@@ -3879,6 +4324,7 @@
       <c r="J421" s="8" t="n"/>
       <c r="K421" s="8" t="n"/>
       <c r="L421" s="8" t="n"/>
+      <c r="M421" s="8" t="n"/>
     </row>
     <row r="422">
       <c r="F422" s="7" t="n"/>
@@ -3886,6 +4332,7 @@
       <c r="J422" s="8" t="n"/>
       <c r="K422" s="8" t="n"/>
       <c r="L422" s="8" t="n"/>
+      <c r="M422" s="8" t="n"/>
     </row>
     <row r="423">
       <c r="F423" s="7" t="n"/>
@@ -3893,6 +4340,7 @@
       <c r="J423" s="8" t="n"/>
       <c r="K423" s="8" t="n"/>
       <c r="L423" s="8" t="n"/>
+      <c r="M423" s="8" t="n"/>
     </row>
     <row r="424">
       <c r="F424" s="7" t="n"/>
@@ -3900,6 +4348,7 @@
       <c r="J424" s="8" t="n"/>
       <c r="K424" s="8" t="n"/>
       <c r="L424" s="8" t="n"/>
+      <c r="M424" s="8" t="n"/>
     </row>
     <row r="425">
       <c r="F425" s="7" t="n"/>
@@ -3907,6 +4356,7 @@
       <c r="J425" s="8" t="n"/>
       <c r="K425" s="8" t="n"/>
       <c r="L425" s="8" t="n"/>
+      <c r="M425" s="8" t="n"/>
     </row>
     <row r="426">
       <c r="F426" s="7" t="n"/>
@@ -3914,6 +4364,7 @@
       <c r="J426" s="8" t="n"/>
       <c r="K426" s="8" t="n"/>
       <c r="L426" s="8" t="n"/>
+      <c r="M426" s="8" t="n"/>
     </row>
     <row r="427">
       <c r="F427" s="7" t="n"/>
@@ -3921,6 +4372,7 @@
       <c r="J427" s="8" t="n"/>
       <c r="K427" s="8" t="n"/>
       <c r="L427" s="8" t="n"/>
+      <c r="M427" s="8" t="n"/>
     </row>
     <row r="428">
       <c r="F428" s="7" t="n"/>
@@ -3928,6 +4380,7 @@
       <c r="J428" s="8" t="n"/>
       <c r="K428" s="8" t="n"/>
       <c r="L428" s="8" t="n"/>
+      <c r="M428" s="8" t="n"/>
     </row>
     <row r="429">
       <c r="F429" s="7" t="n"/>
@@ -3935,6 +4388,7 @@
       <c r="J429" s="8" t="n"/>
       <c r="K429" s="8" t="n"/>
       <c r="L429" s="8" t="n"/>
+      <c r="M429" s="8" t="n"/>
     </row>
     <row r="430">
       <c r="F430" s="7" t="n"/>
@@ -3942,6 +4396,7 @@
       <c r="J430" s="8" t="n"/>
       <c r="K430" s="8" t="n"/>
       <c r="L430" s="8" t="n"/>
+      <c r="M430" s="8" t="n"/>
     </row>
     <row r="431">
       <c r="F431" s="7" t="n"/>
@@ -3949,6 +4404,7 @@
       <c r="J431" s="8" t="n"/>
       <c r="K431" s="8" t="n"/>
       <c r="L431" s="8" t="n"/>
+      <c r="M431" s="8" t="n"/>
     </row>
     <row r="432">
       <c r="F432" s="7" t="n"/>
@@ -3956,6 +4412,7 @@
       <c r="J432" s="8" t="n"/>
       <c r="K432" s="8" t="n"/>
       <c r="L432" s="8" t="n"/>
+      <c r="M432" s="8" t="n"/>
     </row>
     <row r="433">
       <c r="F433" s="7" t="n"/>
@@ -3963,6 +4420,7 @@
       <c r="J433" s="8" t="n"/>
       <c r="K433" s="8" t="n"/>
       <c r="L433" s="8" t="n"/>
+      <c r="M433" s="8" t="n"/>
     </row>
     <row r="434">
       <c r="F434" s="7" t="n"/>
@@ -3970,6 +4428,7 @@
       <c r="J434" s="8" t="n"/>
       <c r="K434" s="8" t="n"/>
       <c r="L434" s="8" t="n"/>
+      <c r="M434" s="8" t="n"/>
     </row>
     <row r="435">
       <c r="F435" s="7" t="n"/>
@@ -3977,6 +4436,7 @@
       <c r="J435" s="8" t="n"/>
       <c r="K435" s="8" t="n"/>
       <c r="L435" s="8" t="n"/>
+      <c r="M435" s="8" t="n"/>
     </row>
     <row r="436">
       <c r="F436" s="7" t="n"/>
@@ -3984,6 +4444,7 @@
       <c r="J436" s="8" t="n"/>
       <c r="K436" s="8" t="n"/>
       <c r="L436" s="8" t="n"/>
+      <c r="M436" s="8" t="n"/>
     </row>
     <row r="437">
       <c r="F437" s="7" t="n"/>
@@ -3991,6 +4452,7 @@
       <c r="J437" s="8" t="n"/>
       <c r="K437" s="8" t="n"/>
       <c r="L437" s="8" t="n"/>
+      <c r="M437" s="8" t="n"/>
     </row>
     <row r="438">
       <c r="F438" s="7" t="n"/>
@@ -3998,6 +4460,7 @@
       <c r="J438" s="8" t="n"/>
       <c r="K438" s="8" t="n"/>
       <c r="L438" s="8" t="n"/>
+      <c r="M438" s="8" t="n"/>
     </row>
     <row r="439">
       <c r="F439" s="7" t="n"/>
@@ -4005,6 +4468,7 @@
       <c r="J439" s="8" t="n"/>
       <c r="K439" s="8" t="n"/>
       <c r="L439" s="8" t="n"/>
+      <c r="M439" s="8" t="n"/>
     </row>
     <row r="440">
       <c r="F440" s="7" t="n"/>
@@ -4012,6 +4476,7 @@
       <c r="J440" s="8" t="n"/>
       <c r="K440" s="8" t="n"/>
       <c r="L440" s="8" t="n"/>
+      <c r="M440" s="8" t="n"/>
     </row>
     <row r="441">
       <c r="F441" s="7" t="n"/>
@@ -4019,6 +4484,7 @@
       <c r="J441" s="8" t="n"/>
       <c r="K441" s="8" t="n"/>
       <c r="L441" s="8" t="n"/>
+      <c r="M441" s="8" t="n"/>
     </row>
     <row r="442">
       <c r="F442" s="7" t="n"/>
@@ -4026,6 +4492,7 @@
       <c r="J442" s="8" t="n"/>
       <c r="K442" s="8" t="n"/>
       <c r="L442" s="8" t="n"/>
+      <c r="M442" s="8" t="n"/>
     </row>
     <row r="443">
       <c r="F443" s="7" t="n"/>
@@ -4033,6 +4500,7 @@
       <c r="J443" s="8" t="n"/>
       <c r="K443" s="8" t="n"/>
       <c r="L443" s="8" t="n"/>
+      <c r="M443" s="8" t="n"/>
     </row>
     <row r="444">
       <c r="F444" s="7" t="n"/>
@@ -4040,6 +4508,7 @@
       <c r="J444" s="8" t="n"/>
       <c r="K444" s="8" t="n"/>
       <c r="L444" s="8" t="n"/>
+      <c r="M444" s="8" t="n"/>
     </row>
     <row r="445">
       <c r="F445" s="7" t="n"/>
@@ -4047,6 +4516,7 @@
       <c r="J445" s="8" t="n"/>
       <c r="K445" s="8" t="n"/>
       <c r="L445" s="8" t="n"/>
+      <c r="M445" s="8" t="n"/>
     </row>
     <row r="446">
       <c r="F446" s="7" t="n"/>
@@ -4054,6 +4524,7 @@
       <c r="J446" s="8" t="n"/>
       <c r="K446" s="8" t="n"/>
       <c r="L446" s="8" t="n"/>
+      <c r="M446" s="8" t="n"/>
     </row>
     <row r="447">
       <c r="F447" s="7" t="n"/>
@@ -4061,6 +4532,7 @@
       <c r="J447" s="8" t="n"/>
       <c r="K447" s="8" t="n"/>
       <c r="L447" s="8" t="n"/>
+      <c r="M447" s="8" t="n"/>
     </row>
     <row r="448">
       <c r="F448" s="7" t="n"/>
@@ -4068,6 +4540,7 @@
       <c r="J448" s="8" t="n"/>
       <c r="K448" s="8" t="n"/>
       <c r="L448" s="8" t="n"/>
+      <c r="M448" s="8" t="n"/>
     </row>
     <row r="449">
       <c r="F449" s="7" t="n"/>
@@ -4075,6 +4548,7 @@
       <c r="J449" s="8" t="n"/>
       <c r="K449" s="8" t="n"/>
       <c r="L449" s="8" t="n"/>
+      <c r="M449" s="8" t="n"/>
     </row>
     <row r="450">
       <c r="F450" s="7" t="n"/>
@@ -4082,6 +4556,7 @@
       <c r="J450" s="8" t="n"/>
       <c r="K450" s="8" t="n"/>
       <c r="L450" s="8" t="n"/>
+      <c r="M450" s="8" t="n"/>
     </row>
     <row r="451">
       <c r="F451" s="7" t="n"/>
@@ -4089,6 +4564,7 @@
       <c r="J451" s="8" t="n"/>
       <c r="K451" s="8" t="n"/>
       <c r="L451" s="8" t="n"/>
+      <c r="M451" s="8" t="n"/>
     </row>
     <row r="452">
       <c r="F452" s="7" t="n"/>
@@ -4096,6 +4572,7 @@
       <c r="J452" s="8" t="n"/>
       <c r="K452" s="8" t="n"/>
       <c r="L452" s="8" t="n"/>
+      <c r="M452" s="8" t="n"/>
     </row>
     <row r="453">
       <c r="F453" s="7" t="n"/>
@@ -4103,6 +4580,7 @@
       <c r="J453" s="8" t="n"/>
       <c r="K453" s="8" t="n"/>
       <c r="L453" s="8" t="n"/>
+      <c r="M453" s="8" t="n"/>
     </row>
     <row r="454">
       <c r="F454" s="7" t="n"/>
@@ -4110,6 +4588,7 @@
       <c r="J454" s="8" t="n"/>
       <c r="K454" s="8" t="n"/>
       <c r="L454" s="8" t="n"/>
+      <c r="M454" s="8" t="n"/>
     </row>
     <row r="455">
       <c r="F455" s="7" t="n"/>
@@ -4117,6 +4596,7 @@
       <c r="J455" s="8" t="n"/>
       <c r="K455" s="8" t="n"/>
       <c r="L455" s="8" t="n"/>
+      <c r="M455" s="8" t="n"/>
     </row>
     <row r="456">
       <c r="F456" s="7" t="n"/>
@@ -4124,6 +4604,7 @@
       <c r="J456" s="8" t="n"/>
       <c r="K456" s="8" t="n"/>
       <c r="L456" s="8" t="n"/>
+      <c r="M456" s="8" t="n"/>
     </row>
     <row r="457">
       <c r="F457" s="7" t="n"/>
@@ -4131,6 +4612,7 @@
       <c r="J457" s="8" t="n"/>
       <c r="K457" s="8" t="n"/>
       <c r="L457" s="8" t="n"/>
+      <c r="M457" s="8" t="n"/>
     </row>
     <row r="458">
       <c r="F458" s="7" t="n"/>
@@ -4138,6 +4620,7 @@
       <c r="J458" s="8" t="n"/>
       <c r="K458" s="8" t="n"/>
       <c r="L458" s="8" t="n"/>
+      <c r="M458" s="8" t="n"/>
     </row>
     <row r="459">
       <c r="F459" s="7" t="n"/>
@@ -4145,6 +4628,7 @@
       <c r="J459" s="8" t="n"/>
       <c r="K459" s="8" t="n"/>
       <c r="L459" s="8" t="n"/>
+      <c r="M459" s="8" t="n"/>
     </row>
     <row r="460">
       <c r="F460" s="7" t="n"/>
@@ -4152,6 +4636,7 @@
       <c r="J460" s="8" t="n"/>
       <c r="K460" s="8" t="n"/>
       <c r="L460" s="8" t="n"/>
+      <c r="M460" s="8" t="n"/>
     </row>
     <row r="461">
       <c r="F461" s="7" t="n"/>
@@ -4159,6 +4644,7 @@
       <c r="J461" s="8" t="n"/>
       <c r="K461" s="8" t="n"/>
       <c r="L461" s="8" t="n"/>
+      <c r="M461" s="8" t="n"/>
     </row>
     <row r="462">
       <c r="F462" s="7" t="n"/>
@@ -4166,6 +4652,7 @@
       <c r="J462" s="8" t="n"/>
       <c r="K462" s="8" t="n"/>
       <c r="L462" s="8" t="n"/>
+      <c r="M462" s="8" t="n"/>
     </row>
     <row r="463">
       <c r="F463" s="7" t="n"/>
@@ -4173,6 +4660,7 @@
       <c r="J463" s="8" t="n"/>
       <c r="K463" s="8" t="n"/>
       <c r="L463" s="8" t="n"/>
+      <c r="M463" s="8" t="n"/>
     </row>
     <row r="464">
       <c r="F464" s="7" t="n"/>
@@ -4180,6 +4668,7 @@
       <c r="J464" s="8" t="n"/>
       <c r="K464" s="8" t="n"/>
       <c r="L464" s="8" t="n"/>
+      <c r="M464" s="8" t="n"/>
     </row>
     <row r="465">
       <c r="F465" s="7" t="n"/>
@@ -4187,6 +4676,7 @@
       <c r="J465" s="8" t="n"/>
       <c r="K465" s="8" t="n"/>
       <c r="L465" s="8" t="n"/>
+      <c r="M465" s="8" t="n"/>
     </row>
     <row r="466">
       <c r="F466" s="7" t="n"/>
@@ -4194,6 +4684,7 @@
       <c r="J466" s="8" t="n"/>
       <c r="K466" s="8" t="n"/>
       <c r="L466" s="8" t="n"/>
+      <c r="M466" s="8" t="n"/>
     </row>
     <row r="467">
       <c r="F467" s="7" t="n"/>
@@ -4201,6 +4692,7 @@
       <c r="J467" s="8" t="n"/>
       <c r="K467" s="8" t="n"/>
       <c r="L467" s="8" t="n"/>
+      <c r="M467" s="8" t="n"/>
     </row>
     <row r="468">
       <c r="F468" s="7" t="n"/>
@@ -4208,6 +4700,7 @@
       <c r="J468" s="8" t="n"/>
       <c r="K468" s="8" t="n"/>
       <c r="L468" s="8" t="n"/>
+      <c r="M468" s="8" t="n"/>
     </row>
     <row r="469">
       <c r="F469" s="7" t="n"/>
@@ -4215,6 +4708,7 @@
       <c r="J469" s="8" t="n"/>
       <c r="K469" s="8" t="n"/>
       <c r="L469" s="8" t="n"/>
+      <c r="M469" s="8" t="n"/>
     </row>
     <row r="470">
       <c r="F470" s="7" t="n"/>
@@ -4222,6 +4716,7 @@
       <c r="J470" s="8" t="n"/>
       <c r="K470" s="8" t="n"/>
       <c r="L470" s="8" t="n"/>
+      <c r="M470" s="8" t="n"/>
     </row>
     <row r="471">
       <c r="F471" s="7" t="n"/>
@@ -4229,6 +4724,7 @@
       <c r="J471" s="8" t="n"/>
       <c r="K471" s="8" t="n"/>
       <c r="L471" s="8" t="n"/>
+      <c r="M471" s="8" t="n"/>
     </row>
     <row r="472">
       <c r="F472" s="7" t="n"/>
@@ -4236,6 +4732,7 @@
       <c r="J472" s="8" t="n"/>
       <c r="K472" s="8" t="n"/>
       <c r="L472" s="8" t="n"/>
+      <c r="M472" s="8" t="n"/>
     </row>
     <row r="473">
       <c r="F473" s="7" t="n"/>
@@ -4243,6 +4740,7 @@
       <c r="J473" s="8" t="n"/>
       <c r="K473" s="8" t="n"/>
       <c r="L473" s="8" t="n"/>
+      <c r="M473" s="8" t="n"/>
     </row>
     <row r="474">
       <c r="F474" s="7" t="n"/>
@@ -4250,6 +4748,7 @@
       <c r="J474" s="8" t="n"/>
       <c r="K474" s="8" t="n"/>
       <c r="L474" s="8" t="n"/>
+      <c r="M474" s="8" t="n"/>
     </row>
     <row r="475">
       <c r="F475" s="7" t="n"/>
@@ -4257,6 +4756,7 @@
       <c r="J475" s="8" t="n"/>
       <c r="K475" s="8" t="n"/>
       <c r="L475" s="8" t="n"/>
+      <c r="M475" s="8" t="n"/>
     </row>
     <row r="476">
       <c r="F476" s="7" t="n"/>
@@ -4264,6 +4764,7 @@
       <c r="J476" s="8" t="n"/>
       <c r="K476" s="8" t="n"/>
       <c r="L476" s="8" t="n"/>
+      <c r="M476" s="8" t="n"/>
     </row>
     <row r="477">
       <c r="F477" s="7" t="n"/>
@@ -4271,6 +4772,7 @@
       <c r="J477" s="8" t="n"/>
       <c r="K477" s="8" t="n"/>
       <c r="L477" s="8" t="n"/>
+      <c r="M477" s="8" t="n"/>
     </row>
     <row r="478">
       <c r="F478" s="7" t="n"/>
@@ -4278,6 +4780,7 @@
       <c r="J478" s="8" t="n"/>
       <c r="K478" s="8" t="n"/>
       <c r="L478" s="8" t="n"/>
+      <c r="M478" s="8" t="n"/>
     </row>
     <row r="479">
       <c r="F479" s="7" t="n"/>
@@ -4285,6 +4788,7 @@
       <c r="J479" s="8" t="n"/>
       <c r="K479" s="8" t="n"/>
       <c r="L479" s="8" t="n"/>
+      <c r="M479" s="8" t="n"/>
     </row>
     <row r="480">
       <c r="F480" s="7" t="n"/>
@@ -4292,6 +4796,7 @@
       <c r="J480" s="8" t="n"/>
       <c r="K480" s="8" t="n"/>
       <c r="L480" s="8" t="n"/>
+      <c r="M480" s="8" t="n"/>
     </row>
     <row r="481">
       <c r="F481" s="7" t="n"/>
@@ -4299,6 +4804,7 @@
       <c r="J481" s="8" t="n"/>
       <c r="K481" s="8" t="n"/>
       <c r="L481" s="8" t="n"/>
+      <c r="M481" s="8" t="n"/>
     </row>
     <row r="482">
       <c r="F482" s="7" t="n"/>
@@ -4306,6 +4812,7 @@
       <c r="J482" s="8" t="n"/>
       <c r="K482" s="8" t="n"/>
       <c r="L482" s="8" t="n"/>
+      <c r="M482" s="8" t="n"/>
     </row>
     <row r="483">
       <c r="F483" s="7" t="n"/>
@@ -4313,6 +4820,7 @@
       <c r="J483" s="8" t="n"/>
       <c r="K483" s="8" t="n"/>
       <c r="L483" s="8" t="n"/>
+      <c r="M483" s="8" t="n"/>
     </row>
     <row r="484">
       <c r="F484" s="7" t="n"/>
@@ -4320,6 +4828,7 @@
       <c r="J484" s="8" t="n"/>
       <c r="K484" s="8" t="n"/>
       <c r="L484" s="8" t="n"/>
+      <c r="M484" s="8" t="n"/>
     </row>
     <row r="485">
       <c r="F485" s="7" t="n"/>
@@ -4327,6 +4836,7 @@
       <c r="J485" s="8" t="n"/>
       <c r="K485" s="8" t="n"/>
       <c r="L485" s="8" t="n"/>
+      <c r="M485" s="8" t="n"/>
     </row>
     <row r="486">
       <c r="F486" s="7" t="n"/>
@@ -4334,6 +4844,7 @@
       <c r="J486" s="8" t="n"/>
       <c r="K486" s="8" t="n"/>
       <c r="L486" s="8" t="n"/>
+      <c r="M486" s="8" t="n"/>
     </row>
     <row r="487">
       <c r="F487" s="7" t="n"/>
@@ -4341,6 +4852,7 @@
       <c r="J487" s="8" t="n"/>
       <c r="K487" s="8" t="n"/>
       <c r="L487" s="8" t="n"/>
+      <c r="M487" s="8" t="n"/>
     </row>
     <row r="488">
       <c r="F488" s="7" t="n"/>
@@ -4348,6 +4860,7 @@
       <c r="J488" s="8" t="n"/>
       <c r="K488" s="8" t="n"/>
       <c r="L488" s="8" t="n"/>
+      <c r="M488" s="8" t="n"/>
     </row>
     <row r="489">
       <c r="F489" s="7" t="n"/>
@@ -4355,6 +4868,7 @@
       <c r="J489" s="8" t="n"/>
       <c r="K489" s="8" t="n"/>
       <c r="L489" s="8" t="n"/>
+      <c r="M489" s="8" t="n"/>
     </row>
     <row r="490">
       <c r="F490" s="7" t="n"/>
@@ -4362,6 +4876,7 @@
       <c r="J490" s="8" t="n"/>
       <c r="K490" s="8" t="n"/>
       <c r="L490" s="8" t="n"/>
+      <c r="M490" s="8" t="n"/>
     </row>
     <row r="491">
       <c r="F491" s="7" t="n"/>
@@ -4369,6 +4884,7 @@
       <c r="J491" s="8" t="n"/>
       <c r="K491" s="8" t="n"/>
       <c r="L491" s="8" t="n"/>
+      <c r="M491" s="8" t="n"/>
     </row>
     <row r="492">
       <c r="F492" s="7" t="n"/>
@@ -4376,6 +4892,7 @@
       <c r="J492" s="8" t="n"/>
       <c r="K492" s="8" t="n"/>
       <c r="L492" s="8" t="n"/>
+      <c r="M492" s="8" t="n"/>
     </row>
     <row r="493">
       <c r="F493" s="7" t="n"/>
@@ -4383,6 +4900,7 @@
       <c r="J493" s="8" t="n"/>
       <c r="K493" s="8" t="n"/>
       <c r="L493" s="8" t="n"/>
+      <c r="M493" s="8" t="n"/>
     </row>
     <row r="494">
       <c r="F494" s="7" t="n"/>
@@ -4390,6 +4908,7 @@
       <c r="J494" s="8" t="n"/>
       <c r="K494" s="8" t="n"/>
       <c r="L494" s="8" t="n"/>
+      <c r="M494" s="8" t="n"/>
     </row>
     <row r="495">
       <c r="F495" s="7" t="n"/>
@@ -4397,6 +4916,7 @@
       <c r="J495" s="8" t="n"/>
       <c r="K495" s="8" t="n"/>
       <c r="L495" s="8" t="n"/>
+      <c r="M495" s="8" t="n"/>
     </row>
     <row r="496">
       <c r="F496" s="7" t="n"/>
@@ -4404,6 +4924,7 @@
       <c r="J496" s="8" t="n"/>
       <c r="K496" s="8" t="n"/>
       <c r="L496" s="8" t="n"/>
+      <c r="M496" s="8" t="n"/>
     </row>
     <row r="497">
       <c r="F497" s="7" t="n"/>
@@ -4411,6 +4932,7 @@
       <c r="J497" s="8" t="n"/>
       <c r="K497" s="8" t="n"/>
       <c r="L497" s="8" t="n"/>
+      <c r="M497" s="8" t="n"/>
     </row>
     <row r="498">
       <c r="F498" s="7" t="n"/>
@@ -4418,6 +4940,7 @@
       <c r="J498" s="8" t="n"/>
       <c r="K498" s="8" t="n"/>
       <c r="L498" s="8" t="n"/>
+      <c r="M498" s="8" t="n"/>
     </row>
     <row r="499">
       <c r="F499" s="7" t="n"/>
@@ -4425,6 +4948,7 @@
       <c r="J499" s="8" t="n"/>
       <c r="K499" s="8" t="n"/>
       <c r="L499" s="8" t="n"/>
+      <c r="M499" s="8" t="n"/>
     </row>
     <row r="500">
       <c r="F500" s="7" t="n"/>
@@ -4432,6 +4956,7 @@
       <c r="J500" s="8" t="n"/>
       <c r="K500" s="8" t="n"/>
       <c r="L500" s="8" t="n"/>
+      <c r="M500" s="8" t="n"/>
     </row>
     <row r="501">
       <c r="F501" s="7" t="n"/>
@@ -4439,11 +4964,12 @@
       <c r="J501" s="8" t="n"/>
       <c r="K501" s="8" t="n"/>
       <c r="L501" s="8" t="n"/>
+      <c r="M501" s="8" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="6">
     <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Modèle absent de la liste : vérifiez qu'il existe dans le back-office (Flotte &gt; Modèles)." type="list" errorStyle="warning">
-      <formula1>=Listes!$A$2:$A$9</formula1>
+      <formula1>=Listes!$A$2:$A$13</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez un statut de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$B$2:$B$5</formula1>
@@ -4451,7 +4977,7 @@
     <dataValidation sqref="E2:E501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez un carburant de la liste." type="list" errorStyle="warning">
       <formula1>=Listes!$C$2:$C$5</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F501 M2:N501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Nombre entier de kilomètres." type="whole" operator="between">
+    <dataValidation sqref="F2:F501 N2:O501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Nombre entier de kilomètres." type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>2000000</formula2>
     </dataValidation>
@@ -4459,7 +4985,7 @@
       <formula1>1990</formula1>
       <formula2>2100</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:L501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Date au format jj/mm/aaaa." type="date" operator="greaterThan">
+    <dataValidation sqref="I2:M501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Date au format jj/mm/aaaa." type="date" operator="greaterThan">
       <formula1>32874</formula1>
     </dataValidation>
   </dataValidations>
@@ -4474,7 +5000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4595,6 +5121,34 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Bentley Continental GTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bentley Bentayga</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Bentley Flying Spur</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Rolls-Royce Cullinan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>